<commit_message>
update fertiliser product data
</commit_message>
<xml_diff>
--- a/Excel/Common_v03.xlsx
+++ b/Excel/Common_v03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{760990C1-2DF8-4D48-ADEF-B4F7F0BC099D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7421B5B6-E3B8-4494-8CF3-E1C9FE3142DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1155" yWindow="465" windowWidth="36255" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="2085" yWindow="1065" windowWidth="36255" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="3" r:id="rId1"/>
@@ -355,7 +355,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="125">
   <si>
     <t>Climate zone</t>
   </si>
@@ -1329,13 +1329,13 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="15">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="14" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="52">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2676,28 +2676,50 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D55AFDDE-E44E-4566-9446-49D22D1085DF}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
-  <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{13023411-FAD9-40B6-9366-7826422CBF8A}" name="Table_Input_DataQuality" displayName="Table_Input_DataQuality" ref="D6:J7" totalsRowShown="0" headerRowCellStyle="Input table column header">
+  <autoFilter ref="D6:J7" xr:uid="{13023411-FAD9-40B6-9366-7826422CBF8A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{8BD56FF8-29E2-4DF7-85A1-55618F035A34}" name="State/Territory">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{A2CDF183-0BAA-498A-9B37-66C6C22B6CF3}" name="Input"/>
+    <tableColumn id="2" xr3:uid="{6CE8517D-1BF5-41D8-AECC-86D1C40836B1}" name="Temporal representativeness" dataCellStyle="Input select"/>
+    <tableColumn id="3" xr3:uid="{C5670EC5-C3E7-45CC-B5CC-F04864805BF9}" name="Spatial resolution" dataCellStyle="Input select"/>
+    <tableColumn id="4" xr3:uid="{7DC7BACF-82BB-4981-857A-7815604920E6}" name="Sample size" dataCellStyle="Input select"/>
+    <tableColumn id="5" xr3:uid="{429BE7C7-3702-4A3D-8940-3720A52AA97C}" name="Notes"/>
+    <tableColumn id="6" xr3:uid="{23695E05-CB90-4B3D-8984-AE8904F2CE28}" name="Evidence files"/>
+    <tableColumn id="7" xr3:uid="{C5FD6441-FC89-47D1-A4AC-0A260329C853}" name="Score" dataCellStyle="Input number general calculated">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Temporal representativeness]],Table_SourceData_DataQuality_TemporalRepresentativeness[ID],Table_SourceData_DataQuality_TemporalRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Spatial resolution]],Table_SourceData_DataQuality_SpatialRepresentativeness[ID],Table_SourceData_DataQuality_SpatialRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Sample size]],Table_SourceData_DataQuality_SampleSize[ID],Table_SourceData_DataQuality_SampleSize[Score])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F5DA0D0E-6BC4-4950-A99F-5113C027644B}" name="Common Name">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+  </tableColumns>
+  <tableStyleInfo name="Editable table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7DB7A349-D3DD-4014-9714-0EE906A80983}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
+  <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{61D54A58-B9CE-4F4F-A6C1-9709184F0C68}" name="Leaching Zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{387B7C9E-D7D9-4D36-A290-1A81ACD3515A}" name="Abbreviation">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{FA4910CF-D781-41C4-A05F-986A4A73D67B}" name="Leaching criteria">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{1BFC15E8-D67C-4277-8EF9-438444043863}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
   <autoFilter ref="D153:E158" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2715,7 +2737,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D871F994-12EC-4014-A3F3-C7F599044252}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2733,7 +2755,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{CFF24A4D-FB3A-4990-A60E-B22F27A25574}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
   <autoFilter ref="D186:H199" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2763,7 +2785,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2781,7 +2803,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
   <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2799,7 +2821,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
   <autoFilter ref="D212:E224" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2817,7 +2839,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
   <autoFilter ref="D231:S250" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2891,7 +2913,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
   <autoFilter ref="D257:E259" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2909,7 +2931,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}" name="Table_SourceData_DataQuality_TemporalRepresentativeness" displayName="Table_SourceData_DataQuality_TemporalRepresentativeness" ref="D265:F270" totalsRowShown="0">
   <autoFilter ref="D265:F270" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2925,7 +2947,29 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D55AFDDE-E44E-4566-9446-49D22D1085DF}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
+  <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{8BD56FF8-29E2-4DF7-85A1-55618F035A34}" name="State/Territory">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{F5DA0D0E-6BC4-4950-A99F-5113C027644B}" name="Common Name">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{387B7C9E-D7D9-4D36-A290-1A81ACD3515A}" name="Abbreviation">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}" name="Table_SourceData_DataQuality_SpatialRepresentativeness" displayName="Table_SourceData_DataQuality_SpatialRepresentativeness" ref="D274:F279" totalsRowShown="0">
   <autoFilter ref="D274:F279" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2941,21 +2985,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B68A2510-6801-4CC4-A35D-1182F8B5B0D6}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
-  <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
-    <filterColumn colId="0" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{FEC43FAA-C4DB-43B0-B971-1FF71C5C3EB9}" name="SA 4 Name">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}" name="Table_SourceData_DataQuality_SampleSize" displayName="Table_SourceData_DataQuality_SampleSize" ref="D283:F288" totalsRowShown="0">
   <autoFilter ref="D283:F288" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2971,7 +3001,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}" name="Table_SourceData_DataQuality_Scope3" displayName="Table_SourceData_DataQuality_Scope3" ref="D292:F297" totalsRowShown="0">
   <autoFilter ref="D292:F297" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2988,6 +3018,20 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B68A2510-6801-4CC4-A35D-1182F8B5B0D6}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
+  <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
+    <filterColumn colId="0" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{FEC43FAA-C4DB-43B0-B971-1FF71C5C3EB9}" name="SA 4 Name">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A8693B4F-0827-4BC0-8BFF-4E2F8802A9A6}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3005,7 +3049,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D62FC099-DF5F-42B5-806A-E7A932074694}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3035,7 +3079,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EFF0180F-7F7D-4433-BEE0-8A0A823637BF}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3109,7 +3153,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{332A6A92-FC29-4D50-BA04-0826843E7703}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3127,7 +3171,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{F9FC6E4B-1485-47B3-B981-452B30BCE51E}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3153,7 +3197,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B7337C26-229C-4E09-A297-90C453C060F3}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3173,24 +3217,6 @@
     </tableColumn>
     <tableColumn id="4" xr3:uid="{9A50E08F-C1E5-4577-BFCD-3512C380DD34}" name="Max rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7DB7A349-D3DD-4014-9714-0EE906A80983}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
-  <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{61D54A58-B9CE-4F4F-A6C1-9709184F0C68}" name="Leaching Zone">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{FA4910CF-D781-41C4-A05F-986A4A73D67B}" name="Leaching criteria">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3548,22 +3574,29 @@
       <c r="I6" s="21" t="s">
         <v>71</v>
       </c>
+      <c r="J6" s="21" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="24">
+        <f>_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Temporal representativeness]],Table_SourceData_DataQuality_TemporalRepresentativeness[ID],Table_SourceData_DataQuality_TemporalRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Spatial resolution]],Table_SourceData_DataQuality_SpatialRepresentativeness[ID],Table_SourceData_DataQuality_SpatialRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Sample size]],Table_SourceData_DataQuality_SampleSize[ID],Table_SourceData_DataQuality_SampleSize[Score])</f>
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -3578,6 +3611,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -7714,68 +7750,68 @@
       </c>
     </row>
     <row r="265" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D265" s="22" t="s">
+      <c r="D265" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E265" s="22" t="s">
+      <c r="E265" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F265" s="22" t="s">
+      <c r="F265" s="11" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="266" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D266" s="22" t="s">
+      <c r="D266" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="E266" s="22" t="s">
+      <c r="E266" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="F266" s="22">
+      <c r="F266" s="11">
         <v>5</v>
       </c>
     </row>
     <row r="267" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D267" s="22" t="s">
+      <c r="D267" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E267" s="22" t="s">
+      <c r="E267" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="F267" s="22">
+      <c r="F267" s="11">
         <v>4</v>
       </c>
     </row>
     <row r="268" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D268" s="22" t="s">
+      <c r="D268" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E268" s="22" t="s">
+      <c r="E268" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="F268" s="22">
+      <c r="F268" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="269" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D269" s="22" t="s">
+      <c r="D269" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="E269" s="22" t="s">
+      <c r="E269" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="F269" s="22">
+      <c r="F269" s="11">
         <v>2</v>
       </c>
     </row>
     <row r="270" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D270" s="22" t="s">
+      <c r="D270" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="E270" s="22" t="s">
+      <c r="E270" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="F270" s="22">
+      <c r="F270" s="11">
         <v>1</v>
       </c>
     </row>
@@ -7785,68 +7821,68 @@
       </c>
     </row>
     <row r="274" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D274" s="22" t="s">
+      <c r="D274" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E274" s="22" t="s">
+      <c r="E274" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F274" s="22" t="s">
+      <c r="F274" s="11" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="275" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D275" s="22" t="s">
+      <c r="D275" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="E275" s="22" t="s">
+      <c r="E275" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="F275" s="22">
+      <c r="F275" s="11">
         <v>5</v>
       </c>
     </row>
     <row r="276" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D276" s="22" t="s">
+      <c r="D276" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E276" s="22" t="s">
+      <c r="E276" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="F276" s="22">
+      <c r="F276" s="11">
         <v>4</v>
       </c>
     </row>
     <row r="277" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D277" s="22" t="s">
+      <c r="D277" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E277" s="22" t="s">
+      <c r="E277" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="F277" s="22">
+      <c r="F277" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="278" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D278" s="22" t="s">
+      <c r="D278" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="E278" s="22" t="s">
+      <c r="E278" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="F278" s="22">
+      <c r="F278" s="11">
         <v>2</v>
       </c>
     </row>
     <row r="279" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D279" s="22" t="s">
+      <c r="D279" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="E279" s="22" t="s">
+      <c r="E279" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="F279" s="22">
+      <c r="F279" s="11">
         <v>1</v>
       </c>
     </row>
@@ -7856,68 +7892,68 @@
       </c>
     </row>
     <row r="283" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D283" s="22" t="s">
+      <c r="D283" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E283" s="22" t="s">
+      <c r="E283" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F283" s="22" t="s">
+      <c r="F283" s="11" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="284" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D284" s="22" t="s">
+      <c r="D284" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E284" s="22" t="s">
+      <c r="E284" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="F284" s="22">
+      <c r="F284" s="11">
         <v>5</v>
       </c>
     </row>
     <row r="285" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D285" s="22" t="s">
+      <c r="D285" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E285" s="22" t="s">
+      <c r="E285" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="F285" s="22">
+      <c r="F285" s="11">
         <v>4</v>
       </c>
     </row>
     <row r="286" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D286" s="22" t="s">
+      <c r="D286" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="E286" s="22" t="s">
+      <c r="E286" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="F286" s="22">
+      <c r="F286" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="287" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D287" s="22" t="s">
+      <c r="D287" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="E287" s="22" t="s">
+      <c r="E287" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F287" s="22">
+      <c r="F287" s="11">
         <v>2</v>
       </c>
     </row>
     <row r="288" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D288" s="22" t="s">
+      <c r="D288" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="E288" s="22" t="s">
+      <c r="E288" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="F288" s="22">
+      <c r="F288" s="11">
         <v>1</v>
       </c>
     </row>
@@ -7927,68 +7963,68 @@
       </c>
     </row>
     <row r="292" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D292" s="22" t="s">
+      <c r="D292" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E292" s="22" t="s">
+      <c r="E292" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F292" s="22" t="s">
+      <c r="F292" s="11" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="293" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D293" s="22" t="s">
+      <c r="D293" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E293" s="22" t="s">
+      <c r="E293" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="F293" s="22">
+      <c r="F293" s="11">
         <v>5</v>
       </c>
     </row>
     <row r="294" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D294" s="22" t="s">
+      <c r="D294" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="E294" s="22" t="s">
+      <c r="E294" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="F294" s="22">
+      <c r="F294" s="11">
         <v>4</v>
       </c>
     </row>
     <row r="295" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D295" s="22" t="s">
+      <c r="D295" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E295" s="22" t="s">
+      <c r="E295" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="F295" s="22">
+      <c r="F295" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="296" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D296" s="22" t="s">
+      <c r="D296" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="E296" s="22" t="s">
+      <c r="E296" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="F296" s="22">
+      <c r="F296" s="11">
         <v>2</v>
       </c>
     </row>
     <row r="297" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D297" s="22" t="s">
+      <c r="D297" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="E297" s="22" t="s">
+      <c r="E297" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="F297" s="22">
+      <c r="F297" s="11">
         <v>1</v>
       </c>
     </row>
@@ -8060,6 +8096,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -8254,31 +8314,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8295,31 +8358,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
remove grazed crop residue
</commit_message>
<xml_diff>
--- a/Excel/Common_v03.xlsx
+++ b/Excel/Common_v03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7421B5B6-E3B8-4494-8CF3-E1C9FE3142DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83DA50F-01CC-4FF8-9136-484FAE7D8BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2085" yWindow="1065" windowWidth="36255" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="36255" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="3" r:id="rId1"/>
@@ -1332,7 +1332,7 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="15">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="14" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="14" applyFont="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="52">
@@ -2546,6 +2546,7 @@
       <sheetName val="Input - Site"/>
       <sheetName val="Input - Enterprise"/>
       <sheetName val="Input - Fert Prod System"/>
+      <sheetName val="Input - Data quality"/>
       <sheetName val="Constants - Common"/>
     </sheetNames>
     <sheetDataSet>
@@ -2606,6 +2607,7 @@
       </sheetData>
       <sheetData sheetId="4"/>
       <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -8096,30 +8098,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -8314,34 +8292,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8358,4 +8333,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
improved text input field identification
</commit_message>
<xml_diff>
--- a/Excel/Common_v03.xlsx
+++ b/Excel/Common_v03.xlsx
@@ -8,39 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83DA50F-01CC-4FF8-9136-484FAE7D8BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D02B3D-251E-42DF-A6F5-804C422883E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="36255" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1395" yWindow="225" windowWidth="37785" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="3" r:id="rId1"/>
-    <sheet name="Input - Data quality" sheetId="5" r:id="rId2"/>
-    <sheet name="Constants - Common" sheetId="2" r:id="rId3"/>
-    <sheet name="Acknowledgements" sheetId="4" r:id="rId4"/>
+    <sheet name="Constants - Common" sheetId="2" r:id="rId2"/>
+    <sheet name="Acknowledgements" sheetId="4" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
+    <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
-    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e" localSheetId="1">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
-    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_LatexEquation">_xlfn.LAMBDA("CO2_e = E_{CH4} \times GWP_{CH4}")</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_NIRReference">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Title">_xlfn.LAMBDA("Convert methane emissions to carbon dioxide equivalent emissions")</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Unit">_xlfn.LAMBDA("t CO2e")</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Variable">_xlfn.LAMBDA("ECH4 CO2e")</definedName>
-    <definedName name="Common_Equations.Common_ConvertN2OToCO2e" localSheetId="1">_xlfn.LAMBDA(_xlpm.E_N2O,_xlpm.GWP_N2O, _xlpm.E_N2O * _xlpm.GWP_N2O)</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e">_xlfn.LAMBDA(_xlpm.E_N2O,_xlpm.GWP_N2O, _xlpm.E_N2O * _xlpm.GWP_N2O)</definedName>
-    <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Arguments" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"EN2O","Nitrous oxide emissions (t N2O)";"GWPN2O","Global warming potential for nitrous oxide (t CO2-e / t N2O)"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"EN2O","Nitrous oxide emissions (t N2O)";"GWPN2O","Global warming potential for nitrous oxide (t CO2-e / t N2O)"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_LatexEquation">_xlfn.LAMBDA("CO2_e = E_{N2O} \times GWP_{N2O}")</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_NIRReference">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Title">_xlfn.LAMBDA("Convert nitrous oxide emissions to carbon dioxide equivalent emissions")</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Unit">_xlfn.LAMBDA("t CO2e")</definedName>
     <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Variable">_xlfn.LAMBDA("EN2O CO2e")</definedName>
-    <definedName name="Common_InputFunctions.Common_GetMCFTemperatureZone" localSheetId="1">_xlfn.LAMBDA(_xlpm.Temperature,_xlpm.MMS,_xlpm.TemperatureArray,_xlpm.MMSArray,_xlpm.ReturnArray, _xlfn.XLOOKUP(MEDIAN(_xlpm.Temperature, MIN(_xlpm.TemperatureArray), MAX(_xlpm.TemperatureArray)), _xlpm.TemperatureArray, _xlfn.XLOOKUP(_xlpm.MMS, _xlpm.MMSArray, _xlpm.ReturnArray)))</definedName>
     <definedName name="Common_InputFunctions.Common_GetMCFTemperatureZone">_xlfn.LAMBDA(_xlpm.Temperature,_xlpm.MMS,_xlpm.TemperatureArray,_xlpm.MMSArray,_xlpm.ReturnArray,
     _xlfn.XLOOKUP(
         MEDIAN(
@@ -52,37 +46,21 @@
         _xlfn.XLOOKUP(_xlpm.MMS, _xlpm.MMSArray, _xlpm.ReturnArray)
     )
 )</definedName>
-    <definedName name="Common_InputFunctions.CommonCropping_GetFracWET" localSheetId="1">_xlfn.LAMBDA(_xlpm.LeachingZone,_xlpm.ProductionSystem,_xlpm.LeachingZoneLookup,_xlpm.LeachingZoneFracWETLookup,_xlpm.ProductionSystemLookup,_xlpm.ProductionSystemFracWETLookup, _xlfn.LET(_xlpm.LeachingZoneFracWET, 'Input - Data quality'!Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.LeachingZone, _xlpm.LeachingZoneLookup, _xlpm.LeachingZoneFracWETLookup), _xlpm.ProductionSystemFracWET, 'Input - Data quality'!Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.ProductionSystem, _xlpm.ProductionSystemLookup, _xlpm.ProductionSystemFracWETLookup), IF(_xlpm.LeachingZoneFracWET + _xlpm.ProductionSystemFracWET &gt; 0, 1, 0)))</definedName>
     <definedName name="Common_InputFunctions.CommonCropping_GetFracWET">_xlfn.LAMBDA(_xlpm.LeachingZone,_xlpm.ProductionSystem,_xlpm.LeachingZoneLookup,_xlpm.LeachingZoneFracWETLookup,_xlpm.ProductionSystemLookup,_xlpm.ProductionSystemFracWETLookup, _xlfn.LET(_xlpm.LeachingZoneFracWET, Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.LeachingZone, _xlpm.LeachingZoneLookup, _xlpm.LeachingZoneFracWETLookup), _xlpm.ProductionSystemFracWET, Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.ProductionSystem, _xlpm.ProductionSystemLookup, _xlpm.ProductionSystemFracWETLookup), IF(_xlpm.LeachingZoneFracWET + _xlpm.ProductionSystemFracWET &gt; 0, 1, 0)))</definedName>
-    <definedName name="Common_InputFunctions.getOverlappingReportingCycles" localSheetId="1">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
     <definedName name="Common_InputFunctions.getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
-    <definedName name="Common_InputFunctions.getOverlappingReportingPeriods" localSheetId="1">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), _xlpm.n, MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1), _xlpm.yrs, _xlfn.SEQUENCE(_xlpm.n, 1, _xlpm.firstYear, 1), _xlpm.starts, DATE(_xlpm.yrs, _xlpm.m, _xlpm.d), _xlpm.ends, _xlfn.MAP(_xlpm.starts, _xlpm.PeriodEnd), _xlpm.tag, IF(_xlpm.starts = _xlpm.ReportingCycleStart, " (This reporting cycle)", ""), _xlpm.startsText, TEXT(_xlpm.starts, "dd mmm yyyy"), _xlpm.endsText, TEXT(_xlpm.ends, "dd mmm yyyy"), _xlpm.rows, IF(_xlpm.n = 0, "", _xlfn.HSTACK(_xlpm.startsText &amp; " to " &amp; _xlpm.endsText &amp; _xlpm.tag)), _xlpm.rows))</definedName>
     <definedName name="Common_InputFunctions.getOverlappingReportingPeriods">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), _xlpm.n, MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1), _xlpm.yrs, _xlfn.SEQUENCE(_xlpm.n, 1, _xlpm.firstYear, 1), _xlpm.starts, DATE(_xlpm.yrs, _xlpm.m, _xlpm.d), _xlpm.ends, _xlfn.MAP(_xlpm.starts, _xlpm.PeriodEnd), _xlpm.tag, IF(_xlpm.starts = _xlpm.ReportingCycleStart, " (This reporting cycle)", ""), _xlpm.startsText, TEXT(_xlpm.starts, "dd mmm yyyy"), _xlpm.endsText, TEXT(_xlpm.ends, "dd mmm yyyy"), IF(_xlpm.n = 0, "", _xlfn.HSTACK(_xlpm.startsText &amp; " to " &amp; _xlpm.endsText &amp; _xlpm.tag))))</definedName>
-    <definedName name="Common_InputFunctions.Utility_ConvertStateCommonNameToAbbreviation" localSheetId="1">_xlfn.LAMBDA(_xlpm.StateCommonName,_xlpm.StateCommonNameArray,_xlpm.StateAbbreviationArray, _xlfn.XLOOKUP(_xlpm.StateCommonName, _xlpm.StateCommonNameArray, _xlpm.StateAbbreviationArray, ""))</definedName>
     <definedName name="Common_InputFunctions.Utility_ConvertStateCommonNameToAbbreviation">_xlfn.LAMBDA(_xlpm.StateCommonName,_xlpm.StateCommonNameArray,_xlpm.StateAbbreviationArray, _xlfn.XLOOKUP(_xlpm.StateCommonName, _xlpm.StateCommonNameArray, _xlpm.StateAbbreviationArray, ""))</definedName>
-    <definedName name="Common_InputFunctions.Utility_DisplayArguments_1_2" localSheetId="1">_xlfn.LAMBDA(_xlpm.ArgumentsArray, _xlfn.CHOOSECOLS(_xlpm.ArgumentsArray, 1, 2))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayArguments_1_2">_xlfn.LAMBDA(_xlpm.ArgumentsArray, _xlfn.CHOOSECOLS(_xlpm.ArgumentsArray, 1, 2))</definedName>
-    <definedName name="Common_InputFunctions.Utility_DisplayArguments_3_4" localSheetId="1">_xlfn.LAMBDA(_xlpm.ArgumentsArray, _xlfn.CHOOSECOLS(_xlpm.ArgumentsArray, 3, 4))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayArguments_3_4">_xlfn.LAMBDA(_xlpm.ArgumentsArray, _xlfn.CHOOSECOLS(_xlpm.ArgumentsArray, 3, 4))</definedName>
-    <definedName name="Common_InputFunctions.Utility_DisplayArrayInTable" localSheetId="1">_xlfn.LAMBDA(_xlpm.ArrayData,_xlpm.TableheaderCell,_xlpm.RowsBetweenHeaderandArray,_xlop.ColumnsBetweenHeaderAndArray, IFERROR(INDEX(_xlfn.UNIQUE(_xlpm.ArrayData), ROW() - 'Input - Data quality'!Common_InputFunctions.Utility_GetArrayTableRowStartNumber(_xlpm.TableheaderCell, _xlpm.RowsBetweenHeaderandArray), COLUMN() - 'Input - Data quality'!Common_InputFunctions.Utility_GetArrayTableColumnStartNumber(_xlpm.TableheaderCell) + IF(_xlfn.ISOMITTED(_xlpm.ColumnsBetweenHeaderAndArray), 1, _xlpm.ColumnsBetweenHeaderAndArray)), ""))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayArrayInTable">_xlfn.LAMBDA(_xlpm.ArrayData,_xlpm.TableheaderCell,_xlpm.RowsBetweenHeaderandArray,_xlop.ColumnsBetweenHeaderAndArray, IFERROR(INDEX(_xlfn.UNIQUE(_xlpm.ArrayData), ROW() - Common_InputFunctions.Utility_GetArrayTableRowStartNumber(_xlpm.TableheaderCell, _xlpm.RowsBetweenHeaderandArray), COLUMN() - Common_InputFunctions.Utility_GetArrayTableColumnStartNumber(_xlpm.TableheaderCell) + IF(_xlfn.ISOMITTED(_xlpm.ColumnsBetweenHeaderAndArray), 1, _xlpm.ColumnsBetweenHeaderAndArray)), ""))</definedName>
-    <definedName name="Common_InputFunctions.Utility_DisplayFunctionName" localSheetId="1">_xlfn.LAMBDA(_xlpm.Function, _xlfn.TEXTBEFORE(_xlfn.FORMULATEXT(_xlpm.Function), "("))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayFunctionName">_xlfn.LAMBDA(_xlpm.Function, _xlfn.TEXTBEFORE(_xlfn.FORMULATEXT(_xlpm.Function), "("))</definedName>
-    <definedName name="Common_InputFunctions.Utility_GetArrayTableColumnStartNumber" localSheetId="1">_xlfn.LAMBDA(_xlpm.TableHeaderCell, COLUMN(_xlpm.TableHeaderCell))</definedName>
     <definedName name="Common_InputFunctions.Utility_GetArrayTableColumnStartNumber">_xlfn.LAMBDA(_xlpm.TableHeaderCell, COLUMN(_xlpm.TableHeaderCell))</definedName>
-    <definedName name="Common_InputFunctions.Utility_GetArrayTableRowStartNumber" localSheetId="1">_xlfn.LAMBDA(_xlpm.TableheaderCell,_xlpm.RowsBetweenHeaderandArray, ROW(_xlpm.TableheaderCell) + _xlpm.RowsBetweenHeaderandArray - 1)</definedName>
     <definedName name="Common_InputFunctions.Utility_GetArrayTableRowStartNumber">_xlfn.LAMBDA(_xlpm.TableheaderCell,_xlpm.RowsBetweenHeaderandArray, ROW(_xlpm.TableheaderCell) + _xlpm.RowsBetweenHeaderandArray - 1)</definedName>
-    <definedName name="Common_InputFunctions.Utility_GetClimateZone" localSheetId="1">_xlfn.LAMBDA(_xlpm.avgTemp,_xlpm.avgRain,_xlpm.frostDays,_xlpm.elev,_xlpm.map_pet,_xlpm.minTempArray,_xlpm.maxTempArray,_xlpm.minRainfallArray,_xlpm.maxRainfallArray,_xlpm.minFrostArray,_xlpm.maxFrostArray,_xlpm.minElevationArray,_xlpm.maxElevationArray,_xlpm.minPETArray,_xlpm.maxPETArray,_xlpm.climateZoneArray, _xlfn.LET(_xlpm.mask, (VALUE(_xlpm.minTempArray) &lt;= _xlpm.avgTemp) * (VALUE(_xlpm.maxTempArray) &gt;= _xlpm.avgTemp) * (VALUE(_xlpm.minRainfallArray) &lt;= _xlpm.avgRain) * (VALUE(_xlpm.maxRainfallArray) &gt;= _xlpm.avgRain) * (VALUE(_xlpm.minFrostArray) &lt;= _xlpm.frostDays) * (VALUE(_xlpm.maxFrostArray) &gt;= _xlpm.frostDays) * (VALUE(_xlpm.minElevationArray) &lt;= _xlpm.elev) * (VALUE(_xlpm.maxElevationArray) &gt;= _xlpm.elev) * (VALUE(_xlpm.minPETArray) &lt;= _xlpm.map_pet) * (VALUE(_xlpm.maxPETArray) &gt;= _xlpm.map_pet), _xlfn.TAKE(_xlfn._xlws.FILTER(_xlpm.climateZoneArray, _xlpm.mask, "No match"), 1)))</definedName>
     <definedName name="Common_InputFunctions.Utility_GetClimateZone">_xlfn.LAMBDA(_xlpm.avgTemp,_xlpm.avgRain,_xlpm.frostDays,_xlpm.elev,_xlpm.map_pet,_xlpm.minTempArray,_xlpm.maxTempArray,_xlpm.minRainfallArray,_xlpm.maxRainfallArray,_xlpm.minFrostArray,_xlpm.maxFrostArray,_xlpm.minElevationArray,_xlpm.maxElevationArray,_xlpm.minPETArray,_xlpm.maxPETArray,_xlpm.climateZoneArray, _xlfn.LET(_xlpm.mask, (VALUE(_xlpm.minTempArray) &lt;= _xlpm.avgTemp) * (VALUE(_xlpm.maxTempArray) &gt;= _xlpm.avgTemp) * (VALUE(_xlpm.minRainfallArray) &lt;= _xlpm.avgRain) * (VALUE(_xlpm.maxRainfallArray) &gt;= _xlpm.avgRain) * (VALUE(_xlpm.minFrostArray) &lt;= _xlpm.frostDays) * (VALUE(_xlpm.maxFrostArray) &gt;= _xlpm.frostDays) * (VALUE(_xlpm.minElevationArray) &lt;= _xlpm.elev) * (VALUE(_xlpm.maxElevationArray) &gt;= _xlpm.elev) * (VALUE(_xlpm.minPETArray) &lt;= _xlpm.map_pet) * (VALUE(_xlpm.maxPETArray) &gt;= _xlpm.map_pet), _xlfn.TAKE(_xlfn._xlws.FILTER(_xlpm.climateZoneArray, _xlpm.mask, "No match"), 1)))</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupItemFromMinMax" localSheetId="1">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.MinArray,_xlpm.MaxArray,_xlpm.ItemArray, _xlfn.LET(_xlpm.mask, (VALUE(_xlpm.MinArray) &lt;= _xlpm.LookupValue) * (VALUE(_xlpm.MaxArray) &gt;= _xlpm.LookupValue), _xlfn._xlws.FILTER(_xlpm.ItemArray, _xlpm.mask, "No match")))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupItemFromMinMax">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.MinArray,_xlpm.MaxArray,_xlpm.ItemArray, _xlfn.LET(_xlpm.mask, (VALUE(_xlpm.MinArray) &lt;= _xlpm.LookupValue) * (VALUE(_xlpm.MaxArray) &gt;= _xlpm.LookupValue), _xlfn._xlws.FILTER(_xlpm.ItemArray, _xlpm.mask, "No match")))</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupN2OEFFromProdIrrigationRainfall" localSheetId="1">_xlfn.LAMBDA(_xlpm.ProductionSystem,_xlpm.IrrigationMethod,_xlpm.RainfallZone,_xlpm.ProductionSystemArray,_xlpm.IrrigationMethodArray,_xlpm.RainfallZoneArray,_xlpm.ReturnArray, _xlfn.LET(_xlpm.IrrigationMethod, IF(_xlpm.IrrigationMethod = "Not irrigated", "Not irrigated", "Any"), _xlpm.RainfallZone, IF(_xlpm.IrrigationMethod = "Not irrigated", _xlpm.RainfallZone, "Any"), _xlfn.XLOOKUP(1, (_xlpm.ProductionSystemArray = _xlpm.ProductionSystem) * (_xlpm.IrrigationMethodArray = _xlpm.IrrigationMethod) * (_xlpm.RainfallZoneArray = _xlpm.RainfallZone), _xlpm.ReturnArray)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupN2OEFFromProdIrrigationRainfall">_xlfn.LAMBDA(_xlpm.ProductionSystem,_xlpm.IrrigationMethod,_xlpm.RainfallZone,_xlpm.ProductionSystemArray,_xlpm.IrrigationMethodArray,_xlpm.RainfallZoneArray,_xlpm.ReturnArray, _xlfn.LET(_xlpm.IrrigationMethod, IF(_xlpm.IrrigationMethod = "Not irrigated", "Not irrigated", "Any"), _xlpm.RainfallZone, IF(_xlpm.IrrigationMethod = "Not irrigated", _xlpm.RainfallZone, "Any"), _xlfn.XLOOKUP(1, (_xlpm.ProductionSystemArray = _xlpm.ProductionSystem) * (_xlpm.IrrigationMethodArray = _xlpm.IrrigationMethod) * (_xlpm.RainfallZoneArray = _xlpm.RainfallZone), _xlpm.ReturnArray)))</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupValueInTable" localSheetId="1">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTable">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""))</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupValueInTableNumber" localSheetId="1">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, IF(ISNUMBER(_xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, "")), _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""), 0))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableNumber">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, IF(ISNUMBER(_xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, "")), _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""), 0))</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupValueInTableOneColumnAndHeader" localSheetId="1">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray,_xlop.ValueIfFalse, IFERROR(_xlfn.XLOOKUP(_xlpm.LookupValue1, _xlpm.LookupArray1, _xlfn.XLOOKUP(_xlpm.LookupValue2, _xlpm.LookupArray2, _xlpm.ReturnArray)), IF(_xlfn.ISOMITTED(_xlpm.ValueIfFalse), "", _xlpm.ValueIfFalse)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableOneColumnAndHeader">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray,_xlop.ValueIfFalse,
     IFERROR(
         _xlfn.XLOOKUP(_xlpm.LookupValue1, _xlpm.LookupArray1,
@@ -91,17 +69,13 @@
         IF(_xlfn.ISOMITTED(_xlpm.ValueIfFalse), "", _xlpm.ValueIfFalse)
     )
 )</definedName>
-    <definedName name="Common_InputFunctions.Utility_LookupValueInTableTwoColumns" localSheetId="1">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray,_xlop.ValueIFFalse, _xlfn.XLOOKUP(1, (_xlpm.LookupArray1 = _xlpm.LookupValue1) * (_xlpm.LookupArray2 = _xlpm.LookupValue2), _xlpm.ReturnArray, IF(_xlfn.ISOMITTED(_xlpm.ValueIFFalse), "", _xlpm.ValueIFFalse)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableTwoColumns">_xlfn.LAMBDA(_xlpm.LookupValue1,_xlpm.LookupValue2,_xlpm.LookupArray1,_xlpm.LookupArray2,_xlpm.ReturnArray,_xlop.ValueIFFalse,
     _xlfn.XLOOKUP(1, (_xlpm.LookupArray1=_xlpm.LookupValue1)*(_xlpm.LookupArray2=_xlpm.LookupValue2), _xlpm.ReturnArray, IF(_xlfn.ISOMITTED(_xlpm.ValueIFFalse), "", _xlpm.ValueIFFalse))
 )</definedName>
-    <definedName name="Common_InputFunctions.Utility_ResultsItemFromEquationTitleAndSource" localSheetId="1">_xlfn.LAMBDA(_xlpm.TitleCell,_xlpm.SourceCell, SUBSTITUTE(LEFT(_xlpm.SourceCell, FIND(",", _xlpm.SourceCell) - 1), "VEERG 2026: ", "") &amp; " " &amp; _xlpm.TitleCell)</definedName>
     <definedName name="Common_InputFunctions.Utility_ResultsItemFromEquationTitleAndSource">_xlfn.LAMBDA(_xlpm.TitleCell,_xlpm.SourceCell,
     SUBSTITUTE(LEFT(_xlpm.SourceCell, FIND(",", _xlpm.SourceCell) -1), "VEERG 2026: ", "") &amp; " " &amp; _xlpm.TitleCell
 )</definedName>
-    <definedName name="Common_InputFunctions.Utility_SourceHyperlink" localSheetId="1">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#'" &amp; _xlpm.sh &amp; "'!" &amp; _xlpm.addr))</definedName>
     <definedName name="Common_InputFunctions.Utility_SourceHyperlink">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#'" &amp; _xlpm.sh &amp; "'!" &amp; _xlpm.addr))</definedName>
-    <definedName name="Common_InputFunctions.Utility_SourceHyperlinkDifferentSheet" localSheetId="1">_xlfn.LAMBDA(_xlpm.TargetCell, _xlfn.LET(_xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"), _xlpm.addr, CELL("address", _xlpm.TargetCell), "#" &amp; _xlpm.addr))</definedName>
     <definedName name="Common_InputFunctions.Utility_SourceHyperlinkDifferentSheet">_xlfn.LAMBDA(_xlpm.TargetCell,
   _xlfn.LET(
     _xlpm.sh, _xlfn.TEXTAFTER(CELL("filename", _xlpm.TargetCell), "]"),
@@ -109,27 +83,20 @@
     "#" &amp; _xlpm.addr
   )
 )</definedName>
-    <definedName name="Common_InputFunctions.Utility_SplitStringIntoArray" localSheetId="1">_xlfn.LAMBDA(_xlpm.Cell,_xlpm.Delimiter,_xlop.CharacterToRemove1,_xlop.CharacterToRemove2, _xlfn.FILTERXML("&lt;t&gt;&lt;s&gt;" &amp; SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlpm.Cell, _xlpm.CharacterToRemove1, ""), _xlpm.CharacterToRemove2, ""), _xlpm.Delimiter, "&lt;/s&gt;&lt;s&gt;") &amp; "&lt;/s&gt;&lt;/t&gt;", "//s"))</definedName>
     <definedName name="Common_InputFunctions.Utility_SplitStringIntoArray">_xlfn.LAMBDA(_xlpm.Cell,_xlpm.Delimiter,_xlop.CharacterToRemove1,_xlop.CharacterToRemove2, _xlfn.FILTERXML("&lt;t&gt;&lt;s&gt;" &amp; SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(_xlpm.Cell, _xlpm.CharacterToRemove1, ""), _xlpm.CharacterToRemove2, ""), _xlpm.Delimiter, "&lt;/s&gt;&lt;s&gt;") &amp; "&lt;/s&gt;&lt;/t&gt;", "//s"))</definedName>
-    <definedName name="Common_InputFunctions.Utility_SumQuantityFromCriteria" localSheetId="1">_xlfn.LAMBDA(_xlpm.Criteria1,_xlpm.Criteria1TypeArray,_xlpm.Quantity,_xlop.Multiplier,_xlop.Criteria2,_xlop.Criteria2Array, _xlfn.LET(_xlpm.multiplier, IF(_xlfn.ISOMITTED(_xlpm.Multiplier), 1, _xlpm.Multiplier), _xlpm.quantity, _xlpm.Quantity * _xlpm.multiplier, _xlpm.criteria1, --(_xlpm.Criteria1TypeArray = _xlpm.Criteria1), _xlpm.criteria2, IF(_xlfn.ISOMITTED(_xlpm.Criteria2), 1, --(_xlpm.Criteria2Array = _xlpm.Criteria2)), SUMPRODUCT(_xlpm.criteria1 * _xlpm.criteria2 * _xlpm.quantity)))</definedName>
     <definedName name="Common_InputFunctions.Utility_SumQuantityFromCriteria">_xlfn.LAMBDA(_xlpm.Criteria1,_xlpm.Criteria1TypeArray,_xlpm.Quantity,_xlop.Multiplier,_xlop.Criteria2,_xlop.Criteria2Array, _xlfn.LET(_xlpm.multiplier, IF(_xlfn.ISOMITTED(_xlpm.Multiplier), 1, _xlpm.Multiplier), _xlpm.quantity, _xlpm.Quantity * _xlpm.multiplier, _xlpm.criteria1, --(_xlpm.Criteria1TypeArray = _xlpm.Criteria1), _xlpm.criteria2, IF(_xlfn.ISOMITTED(_xlpm.Criteria2), 1, --(_xlpm.Criteria2Array = _xlpm.Criteria2)), SUMPRODUCT(_xlpm.criteria1 * _xlpm.criteria2 * _xlpm.quantity)))</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State/Territory","Common Name","Abbreviation";"New South Wales","New South Wales","NSW";"Australian Capital Territory","ACT","ACT";"Victoria","Victoria","VIC";"Queensland","Queensland","QLD";"South Australia","South Australia","SA";"Western Australia","Western Australia","WA";"Tasmania","Tasmania","TAS";"Northern Territory","Northern Territory","NT"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"State/Territory","Common Name","Abbreviation";"New South Wales","New South Wales","NSW";"Australian Capital Territory","ACT","ACT";"Victoria","Victoria","VIC";"Queensland","Queensland","QLD";"South Australia","South Australia","SA";"Western Australia","Western Australia","WA";"Tasmania","Tasmania","TAS";"Northern Territory","Northern Territory","NT"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Source">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Title">_xlfn.LAMBDA("Australian states and territories")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_AustralianStatesTerritories_Variable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Appendices" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Note:";"MAT = mean annual temperature";"MAP = mean annual precipitation";"PET = potential evapotranspiration"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Appendices">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Note:";"MAT = mean annual temperature";"MAP = mean annual precipitation";"PET = potential evapotranspiration"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 16, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate Zone","MAT","MAP","Frost days per year","Elevation","MAP:PET","Min temp","Max temp","Min rainfall","Max rainfall","Min frost days","Max frost days","Min elevation","Max elevation","Min MAP:PET","Min MAP:PET";"Tropical montane","&gt; 18 C","Any","≤ 7","&gt; 1000 m","Any",18.001,999999,-999999,999999,-999999,7,1000,999999,-999999,999999;"Tropical wet","&gt; 18 C","&gt; 2000 mm","≤ 7","≤ 1000 m","Any",18.001,999999,2000.001,999999,-999999,7,-999999,999.999,-999999,999999;"Tropical moist","&gt; 18 C","&gt; 1000 mm - ≤ 2000 mm","≤ 7","≤ 1000 m","Any",18.001,999999,1000.001,2000,-999999,7,-999999,999.999,-999999,999999;"Tropical dry","&gt; 18 C","≤ 1000 mm","≤ 7","≤ 1000 m","Any",18.001,999999,-999999,1000,-999999,7,-999999,999.999,-999999,999999;"Warm temperate moist","&gt; 10 C","Any","Any","Any","&gt; 1",10.001,999999,-999999,999999,-999999,999999,-999999,999999,1.001,999999;"Warm temperate dry","&gt; 10 C","Any","Any","Any","≤ 1",10.001,999999,-999999,999999,-999999,999999,-999999,999999,-999999,1;"Cool temperate moist","&gt; 0 C - ≤ 10 C","Any","Any","Any","&gt; 1",-999999,10,-999999,999999,-999999,999999,-999999,999999,1.001,999999;"Cool temperate dry","&gt; 0 C - ≤ 10 C","Any","Any","Any","≤ 1",-999999,10,-999999,999999,-999999,999999,-999999,999999,-999999,1}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(9, 16, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate Zone","MAT","MAP","Frost days per year","Elevation","MAP:PET","Min temp","Max temp","Min rainfall","Max rainfall","Min frost days","Max frost days","Min elevation","Max elevation","Min MAP:PET","Min MAP:PET";"Tropical montane","&gt; 18 C","Any","≤ 7","&gt; 1000 m","Any",18.001,999999,-999999,999999,-999999,7,1000,999999,-999999,999999;"Tropical wet","&gt; 18 C","&gt; 2000 mm","≤ 7","≤ 1000 m","Any",18.001,999999,2000.001,999999,-999999,7,-999999,999.999,-999999,999999;"Tropical moist","&gt; 18 C","&gt; 1000 mm - ≤ 2000 mm","≤ 7","≤ 1000 m","Any",18.001,999999,1000.001,2000,-999999,7,-999999,999.999,-999999,999999;"Tropical dry","&gt; 18 C","≤ 1000 mm","≤ 7","≤ 1000 m","Any",18.001,999999,-999999,1000,-999999,7,-999999,999.999,-999999,999999;"Warm temperate moist","&gt; 10 C","Any","Any","Any","&gt; 1",10.001,999999,-999999,999999,-999999,999999,-999999,999999,1.001,999999;"Warm temperate dry","&gt; 10 C","Any","Any","Any","≤ 1",10.001,999999,-999999,999999,-999999,999999,-999999,999999,-999999,1;"Cool temperate moist","&gt; 0 C - ≤ 10 C","Any","Any","Any","&gt; 1",-999999,10,-999999,999999,-999999,999999,-999999,999999,1.001,999999;"Cool temperate dry","&gt; 0 C - ≤ 10 C","Any","Any","Any","≤ 1",-999999,10,-999999,999999,-999999,999999,-999999,999999,-999999,1}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Source">_xlfn.LAMBDA("VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Title">_xlfn.LAMBDA("VEERG Australian climate zones")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Variable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Variation" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(5, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo in MAT value for warm temperate dry - changed 10 to 11.";"Added min and max columns for MAT, MAP, frost days per year, elevation, MAP:PET to calculate zones from real climate data.";"GAF accepts rainfall as a proxy for precipitation."}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ClimateZones_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(5, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo in MAT value for warm temperate dry - changed 10 to 11.";"Added min and max columns for MAT, MAP, frost days per year, elevation, MAP:PET to calculate zones from real climate data.";"GAF accepts rainfall as a proxy for precipitation."}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Gas","Conversion factor","Conversion factor 1","Conversion factor 2";"CO2","44/12",44,12;"CH4","16/12",16,12;"N2O","44/28",44,28;"Nox","46/14",46,14;"CO","28/12",28,12;"CO2 Lime","44/12",44,12;"NMVOC","14/12",14,12}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Gas","Conversion factor","Conversion factor 1","Conversion factor 2";"CO2","44/12",44,12;"CH4","16/12",16,12;"N2O","44/28",44,28;"Nox","46/14",46,14;"CO","28/12",28,12;"CO2 Lime","44/12",44,12;"NMVOC","14/12",14,12}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Source">_xlfn.LAMBDA("XXXXXXX")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Title">_xlfn.LAMBDA("Factor to convert elemental mass of gas to molecular mass")</definedName>
@@ -140,7 +107,6 @@
     <definedName name="Common_SourceData.Common_SourceData_ConvertN2oElementalToMolecularCg_Title">_xlfn.LAMBDA("Factor to convert elemental mass of N2O to molecular mass")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ConvertN2oElementalToMolecularCg_Unit">_xlfn.LAMBDA("factor")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_ConvertN2oElementalToMolecularCg_Variable">_xlfn.LAMBDA("CgN2O")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_DataScores_Scope3_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Data source","Data score";"International scope 3 database",1;"Australian scope 3 database",2;"State or regional scope 3 database",3;"Emissions intensity calculated from approved method",4;"Verified credential matching ISO14067",5}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_DataScores_Scope3_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Data source","Data score";"International scope 3 database",1;"Australian scope 3 database",2;"State or regional scope 3 database",3;"Emissions intensity calculated from approved method",4;"Verified credential matching ISO14067",5}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_DataScores_Scope3_Source">_xlfn.LAMBDA("VEERG 2026: XXXXXXXX")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_DataScores_Scope3_Title">_xlfn.LAMBDA("Australian data scores for scope 3")</definedName>
@@ -151,22 +117,18 @@
     <definedName name="Common_SourceData.Common_SourceData_DensityOfMethane_Source">_xlfn.LAMBDA("National Inventory Report 2023 Volume 1: Equations 3.B.1a_2, 3.B.1c_2, 3.B.3_1, 3.B.4g_2")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_DensityOfMethane_Title">_xlfn.LAMBDA("p = density of methane")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_DensityOfMethane_Unit">_xlfn.LAMBDA("kg/m3")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_EFleach_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(1, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"EFleach",0.011}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(1, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"EFleach",0.011}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_NIRReference">_xlfn.LAMBDA("National Inventory Report Volume 1: Equation 3.D.B_10")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Source">_xlfn.LAMBDA("VEERG 2026:5.5.2.3 Constant Parameters")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Title">_xlfn.LAMBDA("Emission factor for nitrogen leaching and runoff")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Unit">_xlfn.LAMBDA("(kg N2O-N / kg N")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Variation">_xlfn.LAMBDA((""))</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_EFN2O_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(15, 5, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Production system j","EFN2O","Production system only","Irrigation method","Rainfall zone";"Irrigated pasture",0.0059,"Pasture","Any","Any";"Irrigated crop",0.007,"Crop","Any","Any";"Non-irrigated pasture",0.0018,"Pasture","Not irrigated","Low rainfall";"Non-irrigated pasture",0.0018,"Pasture","Not irrigated","High rainfall";"Non-irrigated crop (low rainfall)",0.0029,"Crop","Not irrigated","Low rainfall";"Non-irrigated crop (high rainfall)",0.008,"Crop","Not irrigated","High rainfall";"Sugar",0.0199,"Sugar","Any","Any";"Cotton",0.0053,"Cotton","Any","Any";"Horticultural crops",0.0064,"Horticultural crops","Any","Any";"Rice (continuous flooding)",0.003,"Rice","Continuous flooding","Any";"Rice (single and multiple drainage, or alternate wetting and drying)",0.005,"Rice","Single and multiple drainage, or alternate wetting and drying","Any";"Aquaculture",0.0026,"Aquaculture","Any","Any";"Forestry",0.0018,"Forestry","Any","Any"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFN2O_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(15, 5, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Production system j","EFN2O","Production system only","Irrigation method","Rainfall zone";"Irrigated pasture",0.0059,"Pasture","Any","Any";"Irrigated crop",0.007,"Crop","Any","Any";"Non-irrigated pasture",0.0018,"Pasture","Not irrigated","Low rainfall";"Non-irrigated pasture",0.0018,"Pasture","Not irrigated","High rainfall";"Non-irrigated crop (low rainfall)",0.0029,"Crop","Not irrigated","Low rainfall";"Non-irrigated crop (high rainfall)",0.008,"Crop","Not irrigated","High rainfall";"Sugar",0.0199,"Sugar","Any","Any";"Cotton",0.0053,"Cotton","Any","Any";"Horticultural crops",0.0064,"Horticultural crops","Any","Any";"Rice (continuous flooding)",0.003,"Rice","Continuous flooding","Any";"Rice (single and multiple drainage, or alternate wetting and drying)",0.005,"Rice","Single and multiple drainage, or alternate wetting and drying","Any";"Aquaculture",0.0026,"Aquaculture","Any","Any";"Forestry",0.0018,"Forestry","Any","Any"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFN2O_NIRReference">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFN2O_Source">_xlfn.LAMBDA("VEERG 2026: Table A.2.2.1")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFN2O_Title">_xlfn.LAMBDA("Nitrous oxide emission factors for inorganic fertiliser application")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFN2O_Unit">_xlfn.LAMBDA("(kg N2O-N / kg N")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_EFN2O_Variation" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(5, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Removed duplicate 'Aquaculture' row.";"Removed asterisks to aid lookup.";"Added 'production system only', 'rainfall zone' and 'irrigation method' columns to aid lookup.";"Duplicated 'non-irrigated pasture' row with same EF for low and high rainfall zones to aid lookup."}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFN2O_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(5, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Removed duplicate 'Aquaculture' row.";"Removed asterisks to aid lookup.";"Added 'production system only', 'rainfall zone' and 'irrigation method' columns to aid lookup.";"Duplicated 'non-irrigated pasture' row with same EF for low and high rainfall zones to aid lookup."}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate zone","EFNi &amp; EFN2O";"Wet climate zone",0.006;"Dry climate zone",0.005}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate zone","EFNi &amp; EFN2O";"Wet climate zone",0.006;"Dry climate zone",0.005}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_NIRReference">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Source">_xlfn.LAMBDA("VEERG 2026: Table A.2.1.4")</definedName>
@@ -174,87 +136,74 @@
     <definedName name="Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Unit">_xlfn.LAMBDA("kg N2O - N / kg N")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Variable">_xlfn.LAMBDA("EFNi &amp; EFN2Oi")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate zone","EFPRP";"Wet climate zone",0.006;"Dry climate zone",0.002}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate zone","EFPRP";"Wet climate zone",0.006;"Dry climate zone",0.002}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_NIRReference">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Source">_xlfn.LAMBDA("VEERG 2026: Table A.2.2.2")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Title">_xlfn.LAMBDA("Emission factor for urine and dung deposited on pasture, range or paddock")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Unit">_xlfn.LAMBDA("kg N2O - N / kg N")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Variation">_xlfn.LAMBDA("VARIATION FROM SOURCE DATA: Changed 'Dry climate zones' to singular 'Dry climate zone' to aid lookup.")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(1, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"FracLEACH",0.24}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(1, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"FracLEACH",0.24}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_NIRReference">_xlfn.LAMBDA("National Inventory Report Volume 1: Leaching and runoff (3.D.b.2)")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Source">_xlfn.LAMBDA("VEERG 2026:5.5.2.3 Constant Parameters")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Title">_xlfn.LAMBDA("Fraction of N that is available for leaching and runoff")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Unit">_xlfn.LAMBDA("(Dimensionless")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Variation">_xlfn.LAMBDA((""))</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_FracWET_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Is in leaching zone","FracWET";"Yes - in leaching zone",1;"No - not in leaching zone",0}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWET_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Is in leaching zone","FracWET";"Yes - in leaching zone",1;"No - not in leaching zone",0}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWET_NIRReference">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWET_Source">_xlfn.LAMBDA("VEERG 2026:5.5.2.3 Constant Parameters")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWET_Title">_xlfn.LAMBDA("Fraction of N that is available for leaching and runoff")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWET_Unit">_xlfn.LAMBDA("(Dimensionless")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWET_Variation">_xlfn.LAMBDA((""))</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_FracWETIrrigation_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Irrigation type ir","FracWET";"Not irrigated",0;"Drip irrigation",0;"Sprinkler irrigation",1;"Surface irrigation",1;"Other irrigation",1}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWETIrrigation_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Irrigation type ir","FracWET";"Not irrigated",0;"Drip irrigation",0;"Sprinkler irrigation",1;"Surface irrigation",1;"Other irrigation",1}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWETIrrigation_NIRReference">_xlfn.LAMBDA("IPCC 2019 Refinement Volume 4: Chapter 11: N2O Emissions from Managed Soils, and CO2 Emissions from Lime and Urea Application")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWETIrrigation_Source">_xlfn.LAMBDA("VEERG 2026: Chapter 1, section 1.8.2 Leaching, climate and rainfall zones")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWETIrrigation_Title">_xlfn.LAMBDA("FracWET for irrigation types")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWETIrrigation_Unit">_xlfn.LAMBDA("dimensionless")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracWETIrrigation_Variation">_xlfn.LAMBDA("VARIATION FROM SOURCE DATA: Table created based on VEERG text 'Areas are subject to leaching (i.e., in the leaching zone) when... the land is irrigated (except drip irrigation).'")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_GWP_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Gas","CO2-e factor";"CO2",1;"CH4",28;"N2O",265;"CF4",6630;"C2F6",12200;"SF6",22800;"NF3",17200}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_GWP_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(8, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Gas","CO2-e factor";"CO2",1;"CH4",28;"N2O",265;"CF4",6630;"C2F6",12200;"SF6",22800;"NF3",17200}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_GWP_Source">_xlfn.LAMBDA("XXXXXXX")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_GWP_Title">_xlfn.LAMBDA("Global warming potential for greenhouse gases")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_GWP_Unit">_xlfn.LAMBDA("factor")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_GWP_Variable">_xlfn.LAMBDA("GWPN2O")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_LeachingZones_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Leaching Zone","Leaching criteria";"Leaching occurs","Σ(𝑟𝑎𝑖𝑛)&gt;Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦";"Leaching does not occur","Σ(𝑟𝑎𝑖𝑛)≤Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_LeachingZones_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Leaching Zone","Leaching criteria";"Leaching occurs","Σ(𝑟𝑎𝑖𝑛)&gt;Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦";"Leaching does not occur","Σ(𝑟𝑎𝑖𝑛)≤Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_LeachingZones_Source">_xlfn.LAMBDA("VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_LeachingZones_Title">_xlfn.LAMBDA("VEERG Australian leaching zones")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_LeachingZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_LeachingZones_Variable">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_LeachingZones_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_MCFTemperatureZone_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(22, 16, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Temperature zone","MAT (ºC)","Uncovered anerobic lagoon","Covered lagoon","Liquid Slurry (without natural crust)","Daily spread (b)","Composting (passive windrow)","Solid Storage","Pit Storage &lt;1 month","Deep Litter","Poultry Manure (with/without litter)","","Direct processing into pelletized fertiliser","Direct application to soil","Pasture, Range and Paddock (c)(d)","MAT raw";"Cool","≤10",0.66,0.1,0.1,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,10;"Cool",11,0.68,0.1,0.11,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,11;"Cool",12,0.7,0.1,0.13,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,12;"Cool",13,0.71,0.1,0.14,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,13;"Cool",14,0.73,0.1,0.15,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,14;"Temperate",15,0.74,0.1,0.17,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,15;"Temperate",16,0.75,0.1,0.18,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,16;"Temperate",17,0.76,0.1,0.2,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,17;"Temperate",18,0.77,0.1,0.22,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,18;"Temperate",19,0.77,0.1,0.24,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,19;"Temperate",20,0.78,0.1,0.26,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,20;"Temperate",21,0.78,0.1,0.29,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,21;"Temperate",22,0.78,0.1,0.31,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,22;"Temperate",23,0.79,0.1,0.34,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,23;"Temperate",24,0.79,0.1,0.37,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,24;"Temperate",25,0.79,0.1,0.41,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,25;"Warm",26,0.79,0.1,0.44,0.01,0.015,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,26;"Warm",27,0.8,0.1,0.48,0.01,0.015,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,27;"Warm","≥28",0.8,0.1,0.5,0.01,0.015,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,28;"","","Anaerobic lagoon","Digester / covered lagoons","Liquid systems","Daily spread","Composting (passive windrow)","Solid storage","Pit storage","Deep litter","Poultry manure with bedding","Poultry manure without bedding","Direct processing","Direct application","Pasture range and paddock","MAT raw"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MCFTemperatureZone_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(22, 16, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Temperature zone","MAT (ºC)","Uncovered anerobic lagoon","Covered lagoon","Liquid Slurry (without natural crust)","Daily spread (b)","Composting (passive windrow)","Solid Storage","Pit Storage &lt;1 month","Deep Litter","Poultry Manure (with/without litter)","","Direct processing into pelletized fertiliser","Direct application to soil","Pasture, Range and Paddock (c)(d)","MAT raw";"Cool","≤10",0.66,0.1,0.1,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,10;"Cool",11,0.68,0.1,0.11,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,11;"Cool",12,0.7,0.1,0.13,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,12;"Cool",13,0.71,0.1,0.14,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,13;"Cool",14,0.73,0.1,0.15,0.001,0.005,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,14;"Temperate",15,0.74,0.1,0.17,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,15;"Temperate",16,0.75,0.1,0.18,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,16;"Temperate",17,0.76,0.1,0.2,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,17;"Temperate",18,0.77,0.1,0.22,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,18;"Temperate",19,0.77,0.1,0.24,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,19;"Temperate",20,0.78,0.1,0.26,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,20;"Temperate",21,0.78,0.1,0.29,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,21;"Temperate",22,0.78,0.1,0.31,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,22;"Temperate",23,0.79,0.1,0.34,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,23;"Temperate",24,0.79,0.1,0.37,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,24;"Temperate",25,0.79,0.1,0.41,0.005,0.01,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,25;"Warm",26,0.79,0.1,0.44,0.01,0.015,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,26;"Warm",27,0.8,0.1,0.48,0.01,0.015,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,27;"Warm","≥28",0.8,0.1,0.5,0.01,0.015,0.02,0.03,0.04,0.015,0.015,0,0,0.0047,28;"","","Anaerobic lagoon","Digester / covered lagoons","Liquid systems","Daily spread","Composting (passive windrow)","Solid storage","Pit storage","Deep litter","Poultry manure with bedding","Poultry manure without bedding","Direct processing","Direct application","Pasture range and paddock","MAT raw"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MCFTemperatureZone_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.8.1")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MCFTemperatureZone_Title">_xlfn.LAMBDA("Manure Management – Methane conversion factor per temperature zone (fraction) (MCFim)")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MCFTemperatureZone_Unit">_xlfn.LAMBDA("fraction")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MCFTemperatureZone_Variation">_xlfn.LAMBDA("VARIATION FROM SOURCE: Added row of NIR MMA definitions to aid lookup. Duplicated 'Poultry with and without litter' column with separate NIR definitions to aid lookup. Added 'MAT raw' column to allow lookup of numbers.")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_MonthsToSeasons_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(13, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Month","Season";"January","Summer";"February","Summer";"March","Autumn";"April","Autumn";"May","Autumn";"June","Winter";"July","Winter";"August","Winter";"September","Spring";"October","Spring";"November","Spring";"December","Summer"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MonthsToSeasons_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(13, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Month","Season";"January","Summer";"February","Summer";"March","Autumn";"April","Autumn";"May","Autumn";"June","Winter";"July","Winter";"August","Winter";"September","Spring";"October","Spring";"November","Spring";"December","Summer"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MonthsToSeasons_NIRReference">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MonthsToSeasons_Source">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MonthsToSeasons_Title">_xlfn.LAMBDA("Months to Seasons Mapping")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MonthsToSeasons_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_MonthsToSeasons_Variation">_xlfn.LAMBDA("")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_RainfallZones_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Rainfall Zone","Annual rainfall","Rainfall min","Rainfall max";"High rainfall","Annual rainfall &gt; 600mm",600.001,999999;"Low rainfall","Annual rainfall ≤ 600mm",-999999,600}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_RainfallZones_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Rainfall Zone","Annual rainfall","Rainfall min","Rainfall max";"High rainfall","Annual rainfall &gt; 600mm",600.001,999999;"Low rainfall","Annual rainfall ≤ 600mm",-999999,600}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_RainfallZones_Source">_xlfn.LAMBDA("VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_RainfallZones_Title">_xlfn.LAMBDA("VEERG Australian rainfall zones")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_RainfallZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_RainfallZones_Variable">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_RainfallZones_Variation">_xlfn.LAMBDA("VARIATION OF SOURCE DATA: Added extra Rainfall min and Rainfall max columns to calculate zone from real rainfall data.")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_TemperatureZones_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Temperature Zone","Median Annual Temperature (MAT)","Min MAT","Max MAT";"Warm","≥ 26 C",26,999999;"Temperate","15 - 25 C",15,25.999;"Cool","≤ 14 C",-999999,14.999}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_TemperatureZones_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Temperature Zone","Median Annual Temperature (MAT)","Min MAT","Max MAT";"Warm","≥ 26 C",26,999999;"Temperate","15 - 25 C",15,25.999;"Cool","≤ 14 C",-999999,14.999}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_TemperatureZones_Source">_xlfn.LAMBDA("VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_TemperatureZones_Title">_xlfn.LAMBDA("VEERG Australian temperature zones")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_TemperatureZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_TemperatureZones_Variable">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_TemperatureZones_Variation">_xlfn.LAMBDA("VARIATION OF SOURCE DATA: Added extra MAT min and MAT max columns to calculate zone from real temperature data.")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_WASA4Areas_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(11, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"SA 4 Name";"Bunbury";"Mandurah";"Perth - Inner";"Perth - North East";"Perth - North West";"Perth - South East";"Perth - South West";"Western Australia - Wheat Belt";"Western Australia - Outback (North)";"Western Australia - Outback (South)"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WASA4Areas_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(11, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"SA 4 Name";"Bunbury";"Mandurah";"Perth - Inner";"Perth - North East";"Perth - North West";"Perth - South East";"Perth - South West";"Western Australia - Wheat Belt";"Western Australia - Outback (North)";"Western Australia - Outback (South)"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WASA4Areas_Source">_xlfn.LAMBDA("Australian Bureau of Statistics (ABS) - Statistical Areas Level 2 - 2021 - Shapefile")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WASA4Areas_Title">_xlfn.LAMBDA("ABS Statistcal Areas Level 4 - Western Australia")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WASA4Areas_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WASA4Areas_Variable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Data" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(15, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate Zone","Wet or Dry Zone";"Tropical montane","Wet climate zone";"Tropical wet","Wet climate zone";"Tropical moist","Wet climate zone";"Tropical dry","Dry climate zone";"Warm temperate moist","Wet climate zone";"Warm temperate dry","Dry climate zone";"Cool temperate moist","Wet climate zone";"Cool temperate dry","Dry climate zone";"Warm temperate moist - low frost","Wet climate zone";"Warm temperate dry - low frost","Dry climate zone";"Warm temperate moist - high temp","Wet climate zone";"Warm temperate dry - high temp","Dry climate zone";"Cool temperate moist - low frost","Wet climate zone";"Cool temperate dry - low frost","Dry climate zone"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(15, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Climate Zone","Wet or Dry Zone";"Tropical montane","Wet climate zone";"Tropical wet","Wet climate zone";"Tropical moist","Wet climate zone";"Tropical dry","Dry climate zone";"Warm temperate moist","Wet climate zone";"Warm temperate dry","Dry climate zone";"Cool temperate moist","Wet climate zone";"Cool temperate dry","Dry climate zone";"Warm temperate moist - low frost","Wet climate zone";"Warm temperate dry - low frost","Dry climate zone";"Warm temperate moist - high temp","Wet climate zone";"Warm temperate dry - high temp","Dry climate zone";"Cool temperate moist - low frost","Wet climate zone";"Cool temperate dry - low frost","Dry climate zone"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Source">_xlfn.LAMBDA("VEERG 2026: Table 1.2: Translating climate zones to wet and dry zones")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Title">_xlfn.LAMBDA("VEERG Australian wet and dry zones")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variable">_xlfn.LAMBDA("")</definedName>
-    <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variation" localSheetId="1">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo - Changed 'Fry' to 'Dry'."}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo - Changed 'Fry' to 'Dry'."}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData_DensityOfMethane_Data">'Constants - Common'!$D$175</definedName>
     <definedName name="CommonLivestock_InputFunctions.AverageLiveweightEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart,_xlpm.LiveweightAtStart,_xlpm.LiveweightGain, [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) + [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightRemainingAtEndOfMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart, _xlpm.LiveweightAtStart, _xlpm.LiveweightGain))</definedName>
@@ -278,7 +227,6 @@
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonthAddedAndRemaining">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownFromMonthStartTotal(_xlpm.LivestockClass, _xlpm.Month, _xlpm.HeadAtStart) + [0]!CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonth(_xlpm.Month, _xlpm.LivestockClass))</definedName>
     <definedName name="CommonLivestock_SourceData.SourceData_Livestock_Common_SymbolsMMS_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(19, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Symbol","Manure management system","";"1","Anaerobic lagoon","Anaerobic lagoon (m=1)";"2","Liquid systems","Liquid systems (m=2)";"3","Daily spread","Daily spread (m=3)";"3a","Sump and dispersal system","Sump and dispersal system (m=3a)";"3b","Drains to paddock","Drains to paddock (m=3b)";"4","Solid storage","Solid storage (m=4)";"5","Drylot (feed pad)","Drylot (feed pad) (m=5)";"6","Composting (passive windrow)","Composting (passive windrow) (m=6)";"7","Digester / covered lagoons","Digester / covered lagoons (m=7)";"8","Deep litter","Deep litter (m=8)";"9","Pit storage","Pit storage (m=9)";"10","Poultry manure with bedding","Poultry manure with bedding (m=10)";"11","Poultry manure without bedding","Poultry manure without bedding (m=11)";"11a","Belt manure removal","Belt manure removal (m=11a)";"11b","Manure stored in house","Manure stored in house (m=11b)";"12","Direct processing","Direct processing (m=12)";"13","Direct application","Direct application (m=13)";"14","Pasture range and paddock","Pasture range and paddock (m=14)"}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Enterprise_PastureBeef_InputFunctions.multiplyCorrespondingCells">_xlfn.LAMBDA(_xlpm.range1,_xlpm.range2,_xlpm.range3, _xlfn.LET(_xlpm.numRows, ROWS(_xlpm.range1), _xlpm.numCols, COLUMNS(_xlpm.range1), _xlpm.result, _xlfn.MAKEARRAY(_xlpm.numRows, _xlpm.numCols, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, IF(ISNUMBER(INDEX(_xlpm.range1, _xlpm.r, _xlpm.c)), INDEX(_xlpm.range1, _xlpm.r, _xlpm.c), 0) * IF(ISNUMBER(INDEX(_xlpm.range2, _xlpm.r, _xlpm.c)), INDEX(_xlpm.range2, _xlpm.r, _xlpm.c), 0) * IF(ISNUMBER(INDEX(_xlpm.range3, _xlpm.r, _xlpm.c)), INDEX(_xlpm.range3, _xlpm.r, _xlpm.c), 0))), _xlpm.result))</definedName>
-    <definedName name="getOverlappingReportingCycles" localSheetId="1">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingStartMonth,_xlpm.ReportingStartDay, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, _xlpm.ReportingStartMonth, _xlpm.d, _xlpm.ReportingStartDay, _xlpm.A, _xlpm.S - 364, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (DATE(_xlpm.ya, _xlpm.m, _xlpm.d) &lt; _xlpm.A), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
     <definedName name="getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingStartMonth,_xlpm.ReportingStartDay, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, _xlpm.ReportingStartMonth, _xlpm.d, _xlpm.ReportingStartDay, _xlpm.A, _xlpm.S - 364, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (DATE(_xlpm.ya, _xlpm.m, _xlpm.d) &lt; _xlpm.A), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
     <definedName name="InputFunctions_PastureBeef.ConvertMonthlyCalvingToSeason">_xlfn.LAMBDA(_xlpm.Season,_xlpm.SumArray,_xlpm.CalvingMonthArray,_xlpm.MonthArray,_xlpm.MonthToSeasonArray, _xlfn.LET(_xlpm.MonthText, TEXT(_xlpm.CalvingMonthArray, "mmmm"), _xlpm.SeasonPerRow, _xlfn.XLOOKUP(_xlpm.MonthText, _xlpm.MonthArray, _xlpm.MonthToSeasonArray, "", 0), SUM(_xlpm.SumArray * (_xlpm.SeasonPerRow = _xlpm.Season))))</definedName>
     <definedName name="InputFunctions_PastureBeef.LookupLiveweightFromMonth">_xlfn.LAMBDA(_xlpm.State,_xlpm.Region,_xlpm.Month,_xlpm.LivestockClass,_xlpm.StateArray,_xlpm.RegionArray,_xlpm.SeasonArray,_xlpm.LivestockClassArray,_xlpm.ReturnArray,_xlpm.StateCommonNameArray,_xlpm.StateAbbreviationArray,_xlpm.MonthArray,_xlpm.MonthToSeasonArray, _xlfn.LET(_xlpm.Month, TEXT(_xlpm.Month, "mmmm"), _xlpm.State, _xlfn.XLOOKUP(_xlpm.State, _xlpm.StateCommonNameArray, _xlpm.StateAbbreviationArray), _xlpm.Season, _xlfn.XLOOKUP(_xlpm.Month, _xlpm.MonthArray, _xlpm.MonthToSeasonArray), _xlfn.XLOOKUP(1, (_xlpm.StateArray = _xlpm.State) * (_xlpm.RegionArray = _xlpm.Region) * (_xlpm.SeasonArray = _xlpm.Season), _xlfn.XLOOKUP(_xlpm.LivestockClass, _xlpm.LivestockClassArray, _xlpm.ReturnArray))))</definedName>
@@ -355,7 +303,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="117">
   <si>
     <t>Climate zone</t>
   </si>
@@ -564,21 +512,6 @@
     <t>APPENDICES</t>
   </si>
   <si>
-    <t>Input - Data quality</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Evidence files</t>
-  </si>
-  <si>
-    <t>Input</t>
-  </si>
-  <si>
-    <t>Temporal representativeness</t>
-  </si>
-  <si>
     <t>Table_SourceData_DataQuality_TemporalRepresentativeness</t>
   </si>
   <si>
@@ -721,15 +654,6 @@
   </si>
   <si>
     <t>Data quality scoring</t>
-  </si>
-  <si>
-    <t>Spatial resolution</t>
-  </si>
-  <si>
-    <t>Sample size</t>
-  </si>
-  <si>
-    <t>Input name</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1195,7 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
@@ -1320,23 +1244,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="35">
       <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="31">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="32"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="29">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="15">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="14" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="52">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="60">
@@ -2678,50 +2585,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{13023411-FAD9-40B6-9366-7826422CBF8A}" name="Table_Input_DataQuality" displayName="Table_Input_DataQuality" ref="D6:J7" totalsRowShown="0" headerRowCellStyle="Input table column header">
-  <autoFilter ref="D6:J7" xr:uid="{13023411-FAD9-40B6-9366-7826422CBF8A}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D55AFDDE-E44E-4566-9446-49D22D1085DF}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
+  <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
-    <filterColumn colId="3" hiddenButton="1"/>
-    <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A2CDF183-0BAA-498A-9B37-66C6C22B6CF3}" name="Input"/>
-    <tableColumn id="2" xr3:uid="{6CE8517D-1BF5-41D8-AECC-86D1C40836B1}" name="Temporal representativeness" dataCellStyle="Input select"/>
-    <tableColumn id="3" xr3:uid="{C5670EC5-C3E7-45CC-B5CC-F04864805BF9}" name="Spatial resolution" dataCellStyle="Input select"/>
-    <tableColumn id="4" xr3:uid="{7DC7BACF-82BB-4981-857A-7815604920E6}" name="Sample size" dataCellStyle="Input select"/>
-    <tableColumn id="5" xr3:uid="{429BE7C7-3702-4A3D-8940-3720A52AA97C}" name="Notes"/>
-    <tableColumn id="6" xr3:uid="{23695E05-CB90-4B3D-8984-AE8904F2CE28}" name="Evidence files"/>
-    <tableColumn id="7" xr3:uid="{C5FD6441-FC89-47D1-A4AC-0A260329C853}" name="Score" dataCellStyle="Input number general calculated">
-      <calculatedColumnFormula>_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Temporal representativeness]],Table_SourceData_DataQuality_TemporalRepresentativeness[ID],Table_SourceData_DataQuality_TemporalRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Spatial resolution]],Table_SourceData_DataQuality_SpatialRepresentativeness[ID],Table_SourceData_DataQuality_SpatialRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Sample size]],Table_SourceData_DataQuality_SampleSize[ID],Table_SourceData_DataQuality_SampleSize[Score])</calculatedColumnFormula>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{8BD56FF8-29E2-4DF7-85A1-55618F035A34}" name="State/Territory">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Editable table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7DB7A349-D3DD-4014-9714-0EE906A80983}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
-  <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{61D54A58-B9CE-4F4F-A6C1-9709184F0C68}" name="Leaching Zone">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{F5DA0D0E-6BC4-4950-A99F-5113C027644B}" name="Common Name">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{FA4910CF-D781-41C4-A05F-986A4A73D67B}" name="Leaching criteria">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{387B7C9E-D7D9-4D36-A290-1A81ACD3515A}" name="Abbreviation">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{1BFC15E8-D67C-4277-8EF9-438444043863}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D153:E158" totalsRowShown="0">
   <autoFilter ref="D153:E158" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2739,7 +2624,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{D871F994-12EC-4014-A3F3-C7F599044252}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2757,7 +2642,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{CFF24A4D-FB3A-4990-A60E-B22F27A25574}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D186:H199" totalsRowShown="0">
   <autoFilter ref="D186:H199" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2787,7 +2672,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}" name="Table_SourceData_FracWETIrrigation" displayName="Table_SourceData_FracWETIrrigation" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{1F48CA34-50DE-46D5-B32A-BB3A1E818E37}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2805,7 +2690,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}" name="Table_SourceData_EFPastureRangeAndPaddock" displayName="Table_SourceData_EFPastureRangeAndPaddock" ref="D206:E208" totalsRowShown="0">
   <autoFilter ref="D206:E208" xr:uid="{D5BE3F89-D70E-4C53-A71C-E756622DEF38}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2823,7 +2708,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}" name="Table_SourceData_Common_MonthToSeason" displayName="Table_SourceData_Common_MonthToSeason" ref="D212:E224" totalsRowShown="0">
   <autoFilter ref="D212:E224" xr:uid="{97796C3A-D95E-4077-AA20-A8FE4145DAAD}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2841,7 +2726,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}" name="Table_SourceData_Common_MCFTemperatureZone" displayName="Table_SourceData_Common_MCFTemperatureZone" ref="D231:S250" totalsRowShown="0">
   <autoFilter ref="D231:S250" xr:uid="{1D72DD9B-C8FA-48F4-9A11-20231FF87B5A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2915,7 +2800,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}" name="Table_SourceData_Common_EFOrganicFertCropResidues" displayName="Table_SourceData_Common_EFOrganicFertCropResidues" ref="D257:E259" totalsRowShown="0">
   <autoFilter ref="D257:E259" xr:uid="{56E01C14-1BB8-4015-9158-4CEB4D3B605C}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2933,7 +2818,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}" name="Table_SourceData_DataQuality_TemporalRepresentativeness" displayName="Table_SourceData_DataQuality_TemporalRepresentativeness" ref="D265:F270" totalsRowShown="0">
   <autoFilter ref="D265:F270" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2949,29 +2834,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D55AFDDE-E44E-4566-9446-49D22D1085DF}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
-  <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
-    <filterColumn colId="0" hiddenButton="1"/>
-    <filterColumn colId="1" hiddenButton="1"/>
-    <filterColumn colId="2" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{8BD56FF8-29E2-4DF7-85A1-55618F035A34}" name="State/Territory">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{F5DA0D0E-6BC4-4950-A99F-5113C027644B}" name="Common Name">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{387B7C9E-D7D9-4D36-A290-1A81ACD3515A}" name="Abbreviation">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}" name="Table_SourceData_DataQuality_SpatialRepresentativeness" displayName="Table_SourceData_DataQuality_SpatialRepresentativeness" ref="D274:F279" totalsRowShown="0">
   <autoFilter ref="D274:F279" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -2987,7 +2850,21 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B68A2510-6801-4CC4-A35D-1182F8B5B0D6}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
+  <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
+    <filterColumn colId="0" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{FEC43FAA-C4DB-43B0-B971-1FF71C5C3EB9}" name="SA 4 Name">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}" name="Table_SourceData_DataQuality_SampleSize" displayName="Table_SourceData_DataQuality_SampleSize" ref="D283:F288" totalsRowShown="0">
   <autoFilter ref="D283:F288" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3003,7 +2880,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}" name="Table_SourceData_DataQuality_Scope3" displayName="Table_SourceData_DataQuality_Scope3" ref="D292:F297" totalsRowShown="0">
   <autoFilter ref="D292:F297" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3020,20 +2897,6 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B68A2510-6801-4CC4-A35D-1182F8B5B0D6}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
-  <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
-    <filterColumn colId="0" hiddenButton="1"/>
-  </autoFilter>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{FEC43FAA-C4DB-43B0-B971-1FF71C5C3EB9}" name="SA 4 Name">
-      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A8693B4F-0827-4BC0-8BFF-4E2F8802A9A6}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3051,7 +2914,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D62FC099-DF5F-42B5-806A-E7A932074694}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3081,7 +2944,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{EFF0180F-7F7D-4433-BEE0-8A0A823637BF}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3155,7 +3018,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{332A6A92-FC29-4D50-BA04-0826843E7703}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3173,7 +3036,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{F9FC6E4B-1485-47B3-B981-452B30BCE51E}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3199,7 +3062,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B7337C26-229C-4E09-A297-90C453C060F3}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
@@ -3219,6 +3082,24 @@
     </tableColumn>
     <tableColumn id="4" xr3:uid="{9A50E08F-C1E5-4577-BFCD-3512C380DD34}" name="Max rainfall">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7DB7A349-D3DD-4014-9714-0EE906A80983}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
+  <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{61D54A58-B9CE-4F4F-A6C1-9709184F0C68}" name="Leaching Zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{FA4910CF-D781-41C4-A05F-986A4A73D67B}" name="Leaching criteria">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3520,106 +3401,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16C315A-7CC8-4753-9519-BB4446F907F4}">
-  <sheetPr>
-    <tabColor rgb="FFCC6600"/>
-  </sheetPr>
-  <dimension ref="C1:M7"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="49" style="1" customWidth="1"/>
-    <col min="5" max="7" width="30.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="101.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="74.5703125" style="1" customWidth="1"/>
-    <col min="10" max="13" width="30.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="30.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="3:13" s="20" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="C1" s="20" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="3:13" s="8" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="3:13" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-    </row>
-    <row r="6" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D6" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="G6" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="I6" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="J6" s="21" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="3:13" x14ac:dyDescent="0.25">
-      <c r="D7" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="F7" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>112</v>
-      </c>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="24">
-        <f>_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Temporal representativeness]],Table_SourceData_DataQuality_TemporalRepresentativeness[ID],Table_SourceData_DataQuality_TemporalRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Spatial resolution]],Table_SourceData_DataQuality_SpatialRepresentativeness[ID],Table_SourceData_DataQuality_SpatialRepresentativeness[Score])+_xlfn.XLOOKUP(Table_Input_DataQuality[[#This Row],[Sample size]],Table_SourceData_DataQuality_SampleSize[ID],Table_SourceData_DataQuality_SampleSize[Score])</f>
-        <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7" xr:uid="{7AC950BA-B243-4A2B-908C-CE099E570588}">
-      <formula1>INDIRECT("Table_SourceData_DataQuality_TemporalRepresentativeness[ID]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{B4055273-B946-42C8-9570-43C0D83989F4}">
-      <formula1>INDIRECT("Table_SourceData_DataQuality_SpatialRepresentativeness[ID]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G7" xr:uid="{0643B092-4651-4CE2-AF60-342D5FB04D11}">
-      <formula1>INDIRECT("Table_SourceData_DataQuality_SampleSize[ID]")</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83968956-F921-4291-AAEE-DE11952DD430}">
   <sheetPr>
     <tabColor theme="2" tint="-0.499984740745262"/>
@@ -7743,31 +7524,31 @@
     </row>
     <row r="263" spans="4:6" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D263" s="5" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="264" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D264" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="265" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D265" s="11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E265" s="11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F265" s="11" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="266" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D266" s="11" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E266" s="11" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F266" s="11">
         <v>5</v>
@@ -7775,10 +7556,10 @@
     </row>
     <row r="267" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D267" s="11" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E267" s="11" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F267" s="11">
         <v>4</v>
@@ -7786,10 +7567,10 @@
     </row>
     <row r="268" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D268" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E268" s="11" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F268" s="11">
         <v>3</v>
@@ -7797,10 +7578,10 @@
     </row>
     <row r="269" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D269" s="11" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E269" s="11" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="F269" s="11">
         <v>2</v>
@@ -7808,10 +7589,10 @@
     </row>
     <row r="270" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D270" s="11" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E270" s="11" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F270" s="11">
         <v>1</v>
@@ -7819,26 +7600,26 @@
     </row>
     <row r="273" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D273" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="274" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D274" s="11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E274" s="11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F274" s="11" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="275" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D275" s="11" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E275" s="11" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="F275" s="11">
         <v>5</v>
@@ -7846,10 +7627,10 @@
     </row>
     <row r="276" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D276" s="11" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E276" s="11" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="F276" s="11">
         <v>4</v>
@@ -7857,10 +7638,10 @@
     </row>
     <row r="277" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D277" s="11" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E277" s="11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="F277" s="11">
         <v>3</v>
@@ -7868,10 +7649,10 @@
     </row>
     <row r="278" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D278" s="11" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E278" s="11" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F278" s="11">
         <v>2</v>
@@ -7879,10 +7660,10 @@
     </row>
     <row r="279" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D279" s="11" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E279" s="11" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="F279" s="11">
         <v>1</v>
@@ -7890,26 +7671,26 @@
     </row>
     <row r="282" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D282" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="283" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D283" s="11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E283" s="11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F283" s="11" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="284" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D284" s="11" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E284" s="11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="F284" s="11">
         <v>5</v>
@@ -7917,10 +7698,10 @@
     </row>
     <row r="285" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D285" s="11" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E285" s="11" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F285" s="11">
         <v>4</v>
@@ -7928,10 +7709,10 @@
     </row>
     <row r="286" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D286" s="11" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E286" s="11" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="F286" s="11">
         <v>3</v>
@@ -7939,10 +7720,10 @@
     </row>
     <row r="287" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D287" s="11" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="E287" s="11" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F287" s="11">
         <v>2</v>
@@ -7950,10 +7731,10 @@
     </row>
     <row r="288" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D288" s="11" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E288" s="11" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="F288" s="11">
         <v>1</v>
@@ -7961,26 +7742,26 @@
     </row>
     <row r="291" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D291" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="292" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D292" s="11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E292" s="11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F292" s="11" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="293" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D293" s="11" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E293" s="11" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F293" s="11">
         <v>5</v>
@@ -7988,10 +7769,10 @@
     </row>
     <row r="294" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D294" s="11" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E294" s="11" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="F294" s="11">
         <v>4</v>
@@ -7999,10 +7780,10 @@
     </row>
     <row r="295" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D295" s="11" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E295" s="11" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="F295" s="11">
         <v>3</v>
@@ -8010,10 +7791,10 @@
     </row>
     <row r="296" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D296" s="11" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E296" s="11" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F296" s="11">
         <v>2</v>
@@ -8021,10 +7802,10 @@
     </row>
     <row r="297" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D297" s="11" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E297" s="11" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F297" s="11">
         <v>1</v>
@@ -8059,7 +7840,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00F8506-5EB7-47C9-955C-A68351EE5687}">
   <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8293,19 +8074,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -8314,6 +8082,19 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8336,9 +8117,12 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8352,12 +8136,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix remaining excel errors
</commit_message>
<xml_diff>
--- a/Excel/Common_v03.xlsx
+++ b/Excel/Common_v03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCA06CC-240D-4906-91C2-C47421AD96AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4AD98B-3471-4EFC-BE49-75ACD8E87A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="615" yWindow="2340" windowWidth="37785" windowHeight="19140" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="3" r:id="rId1"/>
@@ -307,7 +307,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="138">
   <si>
     <t>Climate zone</t>
   </si>
@@ -658,6 +658,69 @@
   </si>
   <si>
     <t>Data quality scoring</t>
+  </si>
+  <si>
+    <t>User friendly description</t>
+  </si>
+  <si>
+    <t>During this emissions calculation period</t>
+  </si>
+  <si>
+    <t>Within 2 years of this emissions calculation period</t>
+  </si>
+  <si>
+    <t>Within 3 years of this emissions calculation period</t>
+  </si>
+  <si>
+    <t>Within 4 years of this emissions calculation period</t>
+  </si>
+  <si>
+    <t>Unknown, or more than 4 years of this emissions calculation period</t>
+  </si>
+  <si>
+    <t>This location with spatial partitioning</t>
+  </si>
+  <si>
+    <t>This location without spatial partitioning</t>
+  </si>
+  <si>
+    <t>Regional-level data from a government or industry database/survey</t>
+  </si>
+  <si>
+    <t>State-level data from a government or industry database/survey</t>
+  </si>
+  <si>
+    <t>National-level data from a government or industry database/survey</t>
+  </si>
+  <si>
+    <t>Over 90%</t>
+  </si>
+  <si>
+    <t>Between 51% and 90%</t>
+  </si>
+  <si>
+    <t>Between 21% and 50%</t>
+  </si>
+  <si>
+    <t>Less than 20%</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Verified report complying to ISO14067 2018 or GHG Protocol Lifecycle Accounting and Reporting Standard</t>
+  </si>
+  <si>
+    <t>Report consistent with ISO14067 2018, GHG Protocol Lifecycle Accounting and Reporting Standard or this tool</t>
+  </si>
+  <si>
+    <t>Regional-level database</t>
+  </si>
+  <si>
+    <t>National-level database</t>
+  </si>
+  <si>
+    <t>Geographically generic database</t>
   </si>
 </sst>
 </file>
@@ -1312,7 +1375,103 @@
     <cellStyle name="Unit no indent" xfId="53" xr:uid="{2829D020-DAD8-4B7D-9262-450720E27D2B}"/>
     <cellStyle name="Unit total" xfId="25" xr:uid="{65428923-3DAD-47B6-8DDF-0EBD05E7C55B}"/>
   </cellStyles>
-  <dxfs count="49">
+  <dxfs count="53">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2403,20 +2562,20 @@
   </dxfs>
   <tableStyles count="3" defaultTableStyle="Equation table" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Editable table" pivot="0" count="6" xr9:uid="{8C498A1C-5864-4BF8-8739-A3055FE117E0}">
-      <tableStyleElement type="wholeTable" dxfId="48"/>
-      <tableStyleElement type="headerRow" dxfId="47"/>
-      <tableStyleElement type="totalRow" dxfId="46"/>
-      <tableStyleElement type="firstColumn" dxfId="45"/>
-      <tableStyleElement type="firstRowStripe" dxfId="44"/>
-      <tableStyleElement type="secondRowStripe" dxfId="43"/>
+      <tableStyleElement type="wholeTable" dxfId="52"/>
+      <tableStyleElement type="headerRow" dxfId="51"/>
+      <tableStyleElement type="totalRow" dxfId="50"/>
+      <tableStyleElement type="firstColumn" dxfId="49"/>
+      <tableStyleElement type="firstRowStripe" dxfId="48"/>
+      <tableStyleElement type="secondRowStripe" dxfId="47"/>
     </tableStyle>
     <tableStyle name="Equation table" pivot="0" count="6" xr9:uid="{B247698E-E41D-4CCD-AA0A-C14817E9DE65}">
-      <tableStyleElement type="wholeTable" dxfId="42"/>
-      <tableStyleElement type="headerRow" dxfId="41"/>
-      <tableStyleElement type="totalRow" dxfId="40"/>
-      <tableStyleElement type="firstColumn" dxfId="39"/>
-      <tableStyleElement type="firstRowStripe" dxfId="38"/>
-      <tableStyleElement type="secondRowStripe" dxfId="37"/>
+      <tableStyleElement type="wholeTable" dxfId="46"/>
+      <tableStyleElement type="headerRow" dxfId="45"/>
+      <tableStyleElement type="totalRow" dxfId="44"/>
+      <tableStyleElement type="firstColumn" dxfId="43"/>
+      <tableStyleElement type="firstRowStripe" dxfId="42"/>
+      <tableStyleElement type="secondRowStripe" dxfId="41"/>
     </tableStyle>
     <tableStyle name="Table Style 1" pivot="0" count="0" xr9:uid="{97B370DB-5463-4A31-9160-5A96BD6A559D}"/>
   </tableStyles>
@@ -2559,7 +2718,7 @@
     <tableColumn id="1" xr3:uid="{CA74DB79-CAE7-4EF8-BA48-96421E9E9373}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F0DDE0C3-8378-485B-A4A4-D07B38ADF801}" name="FracWET" dataDxfId="20">
+    <tableColumn id="2" xr3:uid="{F0DDE0C3-8378-485B-A4A4-D07B38ADF801}" name="FracWET" dataDxfId="24">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2607,7 +2766,7 @@
     <tableColumn id="1" xr3:uid="{B18D772B-2FE9-457A-A200-8E17C55C340C}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A11A4C1D-EDEC-4818-93B7-672872C6D107}" name="FracWET" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{A11A4C1D-EDEC-4818-93B7-672872C6D107}" name="FracWET" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2625,7 +2784,7 @@
     <tableColumn id="1" xr3:uid="{718360C9-DDF8-4B7B-B842-EE0D39ED743F}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{876E0F1A-E7CF-4E69-9C3F-6E0E84FF4B5D}" name="EFPRP" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{876E0F1A-E7CF-4E69-9C3F-6E0E84FF4B5D}" name="EFPRP" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2643,7 +2802,7 @@
     <tableColumn id="1" xr3:uid="{7CBE043C-4D22-47C3-AE18-5E55E64542E1}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{10DA8C9D-4358-470A-AF6C-AE27470313DE}" name="Season" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{10DA8C9D-4358-470A-AF6C-AE27470313DE}" name="Season" dataDxfId="21" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2675,49 +2834,49 @@
     <tableColumn id="1" xr3:uid="{8E03AF9F-C6DD-415E-A42C-F2360BC32F72}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{07B3EB32-B4EC-4553-A2E1-8AE19F5ED1B8}" name="MAT (ºC)" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{07B3EB32-B4EC-4553-A2E1-8AE19F5ED1B8}" name="MAT (ºC)" dataDxfId="20" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{D245CE73-83DF-4AB6-BE51-10D787832614}" name="Anaerobic lagoon" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{D245CE73-83DF-4AB6-BE51-10D787832614}" name="Anaerobic lagoon" dataDxfId="19" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{96977D75-8628-4103-9D52-F7049CB2572B}" name="Digester / covered lagoons" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{96977D75-8628-4103-9D52-F7049CB2572B}" name="Digester / covered lagoons" dataDxfId="18" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{F64B281A-2EA4-4881-94F1-FEBD2B18C677}" name="Liquid systems" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{F64B281A-2EA4-4881-94F1-FEBD2B18C677}" name="Liquid systems" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8934BA44-DDF5-433B-A89F-5DB281BAB7B5}" name="Daily spread" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{8934BA44-DDF5-433B-A89F-5DB281BAB7B5}" name="Daily spread" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{699EC0ED-651C-48B9-9F8F-73146B12DB72}" name="Composting (passive windrow)" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{699EC0ED-651C-48B9-9F8F-73146B12DB72}" name="Composting (passive windrow)" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{6E240578-9A8B-47C9-A356-B69BB058D44B}" name="Solid storage" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{6E240578-9A8B-47C9-A356-B69BB058D44B}" name="Solid storage" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{922DD34E-8EDF-42D6-BE68-8D30A5F4A8CF}" name="Pit storage" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{922DD34E-8EDF-42D6-BE68-8D30A5F4A8CF}" name="Pit storage" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{730FA508-F44F-43A0-8A87-F28C2DB6D4D5}" name="Deep litter" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{730FA508-F44F-43A0-8A87-F28C2DB6D4D5}" name="Deep litter" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{8BD6E90D-D2CF-4733-8286-F67C28172389}" name="Poultry manure with bedding" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{8BD6E90D-D2CF-4733-8286-F67C28172389}" name="Poultry manure with bedding" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{EE74F5BC-4374-40FF-85F0-AE26E403B07E}" name="Poultry manure without bedding" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{EE74F5BC-4374-40FF-85F0-AE26E403B07E}" name="Poultry manure without bedding" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{B53034D9-4966-41B7-BD99-44BBB861677D}" name="Direct processing" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{B53034D9-4966-41B7-BD99-44BBB861677D}" name="Direct processing" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{59F06DF1-1149-43CE-9ADC-FD2C1D44B8D0}" name="Direct application" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{59F06DF1-1149-43CE-9ADC-FD2C1D44B8D0}" name="Direct application" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{E8CF9642-D223-420C-B387-277C82D3BB2E}" name="Pasture range and paddock" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{E8CF9642-D223-420C-B387-277C82D3BB2E}" name="Pasture range and paddock" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{0B403FCE-8D29-4E28-99ED-B0004709790F}" name="MAT raw" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{0B403FCE-8D29-4E28-99ED-B0004709790F}" name="MAT raw" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2735,7 +2894,7 @@
     <tableColumn id="1" xr3:uid="{3C12381E-3675-4A77-B50C-CAF33F1781C7}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{15B1FB4A-EB78-4095-8978-98D149B427BD}" name="EFNi &amp; EFN2Oi" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{15B1FB4A-EB78-4095-8978-98D149B427BD}" name="EFNi &amp; EFN2Oi" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2744,14 +2903,16 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}" name="Table_SourceData_DataQuality_TemporalRepresentativeness" displayName="Table_SourceData_DataQuality_TemporalRepresentativeness" ref="D265:F270" totalsRowShown="0">
-  <autoFilter ref="D265:F270" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}" name="Table_SourceData_DataQuality_TemporalRepresentativeness" displayName="Table_SourceData_DataQuality_TemporalRepresentativeness" ref="D265:G270" totalsRowShown="0">
+  <autoFilter ref="D265:G270" xr:uid="{9AD44602-D2F2-4D97-923C-A32E98F8C17A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{EEF9FA42-D387-4999-8DA3-0AB968DE5B49}" name="Description" dataDxfId="0" dataCellStyle="Content normal"/>
+  <tableColumns count="4">
+    <tableColumn id="4" xr3:uid="{FEABA93E-2C84-4F8B-AD41-9A8E420FF89F}" name="User friendly description" dataDxfId="3" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{EEF9FA42-D387-4999-8DA3-0AB968DE5B49}" name="Description" dataDxfId="4" dataCellStyle="Content normal"/>
     <tableColumn id="1" xr3:uid="{AB1526C9-DA24-4CC9-B5EF-21A0F80180A1}" name="ID"/>
     <tableColumn id="3" xr3:uid="{2DA8D021-3344-47CC-9BAF-CCD2982CBA69}" name="Score"/>
   </tableColumns>
@@ -2760,13 +2921,15 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}" name="Table_SourceData_DataQuality_SpatialRepresentativeness" displayName="Table_SourceData_DataQuality_SpatialRepresentativeness" ref="D274:F279" totalsRowShown="0">
-  <autoFilter ref="D274:F279" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}" name="Table_SourceData_DataQuality_SpatialRepresentativeness" displayName="Table_SourceData_DataQuality_SpatialRepresentativeness" ref="D274:G279" totalsRowShown="0">
+  <autoFilter ref="D274:G279" xr:uid="{95094D65-3E0E-45CE-A3F4-F41E74C11901}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="3">
+  <tableColumns count="4">
+    <tableColumn id="4" xr3:uid="{8F6174C3-89C3-4B10-86C2-6A31851B07A4}" name="User friendly description" dataDxfId="2" dataCellStyle="Content normal"/>
     <tableColumn id="1" xr3:uid="{1849C441-004D-43F7-9536-F4D3575BC03A}" name="Description"/>
     <tableColumn id="2" xr3:uid="{2EA84693-0D7E-4E6D-A008-71E4D387FE32}" name="ID"/>
     <tableColumn id="3" xr3:uid="{0F873D1E-9AF5-43C5-A381-3F4760BB41BF}" name="Score"/>
@@ -2790,13 +2953,15 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}" name="Table_SourceData_DataQuality_SampleSize" displayName="Table_SourceData_DataQuality_SampleSize" ref="D283:F288" totalsRowShown="0">
-  <autoFilter ref="D283:F288" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}" name="Table_SourceData_DataQuality_SampleSize" displayName="Table_SourceData_DataQuality_SampleSize" ref="D283:G288" totalsRowShown="0">
+  <autoFilter ref="D283:G288" xr:uid="{DE8F748C-E65A-4AA2-81BB-D28A432CF334}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="3">
+  <tableColumns count="4">
+    <tableColumn id="4" xr3:uid="{09186B8A-5E2A-49CD-8802-3F9B0F7EC226}" name="User friendly description" dataDxfId="1" dataCellStyle="Content normal"/>
     <tableColumn id="1" xr3:uid="{EB2D29FA-8BB9-4C96-B01A-C17C52C76465}" name="Description"/>
     <tableColumn id="2" xr3:uid="{DC813F48-FE91-49F9-951B-D509D706CF09}" name="ID"/>
     <tableColumn id="3" xr3:uid="{DD670A12-0EA9-4344-8058-F7F57417108F}" name="Score"/>
@@ -2806,13 +2971,15 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}" name="Table_SourceData_DataQuality_Scope3" displayName="Table_SourceData_DataQuality_Scope3" ref="D292:F297" totalsRowShown="0">
-  <autoFilter ref="D292:F297" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}" name="Table_SourceData_DataQuality_Scope3" displayName="Table_SourceData_DataQuality_Scope3" ref="D292:G297" totalsRowShown="0">
+  <autoFilter ref="D292:G297" xr:uid="{43A1C4DA-75D1-45DF-BA9A-1798C2CC5A4B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="3">
+  <tableColumns count="4">
+    <tableColumn id="4" xr3:uid="{8403EC01-6798-45E2-B51A-4AF99E10C45A}" name="User friendly description" dataDxfId="0" dataCellStyle="Content normal"/>
     <tableColumn id="1" xr3:uid="{375B2CFE-E727-4795-9B4F-05A1E0DC4AED}" name="Description"/>
     <tableColumn id="2" xr3:uid="{830FB755-D404-43AF-922A-796F2CCAEA50}" name="ID"/>
     <tableColumn id="3" xr3:uid="{15047EEC-A818-4168-BABD-BB70ACD6159D}" name="Score"/>
@@ -2893,49 +3060,49 @@
     <tableColumn id="1" xr3:uid="{8938BBE8-7B92-48A9-872B-3320D21DB635}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{658207C9-89A7-4F8D-BFB1-8E32C6E5CE10}" name="MAT" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{658207C9-89A7-4F8D-BFB1-8E32C6E5CE10}" name="MAT" totalsRowDxfId="40" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{354F10CE-DC7A-49A5-AA19-EEB6281A6412}" name="MAP" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{354F10CE-DC7A-49A5-AA19-EEB6281A6412}" name="MAP" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{38F4182B-B4B5-426D-98BC-0B2593A7B2AC}" name="Frost days per year" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{38F4182B-B4B5-426D-98BC-0B2593A7B2AC}" name="Frost days per year" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{EE15735E-8ABF-428C-B015-3F1955A6D060}" name="Elevation" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{EE15735E-8ABF-428C-B015-3F1955A6D060}" name="Elevation" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{24D889BF-3FFC-47F8-87FE-E95F033D2601}" name="MAP:PET" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{24D889BF-3FFC-47F8-87FE-E95F033D2601}" name="MAP:PET" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{8B1AA507-6E86-4E0A-8123-6045EBFC43F0}" name="Min temp" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{8B1AA507-6E86-4E0A-8123-6045EBFC43F0}" name="Min temp" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B7A64A9C-167B-48BE-9126-A0FC1AEC24A5}" name="Max temp" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{B7A64A9C-167B-48BE-9126-A0FC1AEC24A5}" name="Max temp" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{6A8CA332-9832-49EA-97FB-DD23C730245E}" name="Min rainfall" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{6A8CA332-9832-49EA-97FB-DD23C730245E}" name="Min rainfall" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{B24E0786-86EC-449C-85EE-60C753B18536}" name="Max rainfall" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{B24E0786-86EC-449C-85EE-60C753B18536}" name="Max rainfall" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{25C5B38E-3202-4F57-A055-5B1AD8BE4CEF}" name="Min frost days" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{25C5B38E-3202-4F57-A055-5B1AD8BE4CEF}" name="Min frost days" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{E486BEC3-9016-4BF3-8FB0-8F4450C55190}" name="Max frost days" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{E486BEC3-9016-4BF3-8FB0-8F4450C55190}" name="Max frost days" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{8C9D6103-6384-43E4-AD6A-556A38AB52A4}" name="Min elevation" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{8C9D6103-6384-43E4-AD6A-556A38AB52A4}" name="Min elevation" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{BF7FD137-AA7E-444B-8D18-DC8AB8FE4C1A}" name="Max elevation" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{BF7FD137-AA7E-444B-8D18-DC8AB8FE4C1A}" name="Max elevation" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{99EBF2EA-96A6-4345-93B0-3364616813EA}" name="Min MAP:PET" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{99EBF2EA-96A6-4345-93B0-3364616813EA}" name="Min MAP:PET" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{3EB0AAD6-2B47-4B1F-AB9F-DF46F10D5123}" name="Max MAP:PET" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{3EB0AAD6-2B47-4B1F-AB9F-DF46F10D5123}" name="Max MAP:PET" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2953,7 +3120,7 @@
     <tableColumn id="1" xr3:uid="{2FCD4A06-823B-4A3F-89D0-46C27A9E1AA9}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{605D6DF8-71A8-491A-BF4E-F6D008835D65}" name="Wet or Dry Zone" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{605D6DF8-71A8-491A-BF4E-F6D008835D65}" name="Wet or Dry Zone" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7419,7 +7586,7 @@
         <v>kg N2O - N / kg N</v>
       </c>
     </row>
-    <row r="257" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="257" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D257" s="11" t="s">
         <v>66</v>
       </c>
@@ -7427,7 +7594,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="258" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="258" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D258" s="11" t="str" cm="1">
         <f t="array" ref="D258">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</f>
         <v>Wet climate zone</v>
@@ -7437,7 +7604,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="259" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="259" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D259" s="1" t="str" cm="1">
         <f t="array" ref="D259">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</f>
         <v>Dry climate zone</v>
@@ -7447,294 +7614,414 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="263" spans="4:6" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="263" spans="4:66" ht="23.25" x14ac:dyDescent="0.25">
       <c r="D263" s="5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="264" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="264" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D264" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="265" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="265" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D265" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E265" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E265" s="11" t="s">
+      <c r="F265" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F265" s="11" t="s">
+      <c r="G265" s="11" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="266" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V265" s="1"/>
+      <c r="BN265" s="6"/>
+    </row>
+    <row r="266" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D266" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E266" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="E266" s="11" t="s">
+      <c r="F266" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="F266" s="11">
+      <c r="G266" s="11">
         <v>5</v>
       </c>
-    </row>
-    <row r="267" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V266" s="1"/>
+      <c r="BN266" s="6"/>
+    </row>
+    <row r="267" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D267" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E267" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="E267" s="11" t="s">
+      <c r="F267" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F267" s="11">
+      <c r="G267" s="11">
         <v>4</v>
       </c>
-    </row>
-    <row r="268" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V267" s="1"/>
+      <c r="BN267" s="6"/>
+    </row>
+    <row r="268" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D268" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="E268" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E268" s="11" t="s">
+      <c r="F268" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F268" s="11">
+      <c r="G268" s="11">
         <v>3</v>
       </c>
-    </row>
-    <row r="269" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V268" s="1"/>
+      <c r="BN268" s="6"/>
+    </row>
+    <row r="269" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D269" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="E269" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="E269" s="11" t="s">
+      <c r="F269" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="F269" s="11">
+      <c r="G269" s="11">
         <v>2</v>
       </c>
-    </row>
-    <row r="270" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V269" s="1"/>
+      <c r="BN269" s="6"/>
+    </row>
+    <row r="270" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D270" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="E270" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E270" s="11" t="s">
+      <c r="F270" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="F270" s="11">
+      <c r="G270" s="11">
         <v>1</v>
       </c>
-    </row>
-    <row r="273" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V270" s="1"/>
+      <c r="BN270" s="6"/>
+    </row>
+    <row r="273" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D273" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="274" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="274" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D274" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E274" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E274" s="11" t="s">
+      <c r="F274" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F274" s="11" t="s">
+      <c r="G274" s="11" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="275" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V274" s="1"/>
+      <c r="BN274" s="6"/>
+    </row>
+    <row r="275" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D275" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E275" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="E275" s="11" t="s">
+      <c r="F275" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="F275" s="11">
+      <c r="G275" s="11">
         <v>5</v>
       </c>
-    </row>
-    <row r="276" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V275" s="1"/>
+      <c r="BN275" s="6"/>
+    </row>
+    <row r="276" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D276" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E276" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="E276" s="11" t="s">
+      <c r="F276" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F276" s="11">
+      <c r="G276" s="11">
         <v>4</v>
       </c>
-    </row>
-    <row r="277" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V276" s="1"/>
+      <c r="BN276" s="6"/>
+    </row>
+    <row r="277" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D277" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="E277" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E277" s="11" t="s">
+      <c r="F277" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="F277" s="11">
+      <c r="G277" s="11">
         <v>3</v>
       </c>
-    </row>
-    <row r="278" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V277" s="1"/>
+      <c r="BN277" s="6"/>
+    </row>
+    <row r="278" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D278" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E278" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="E278" s="11" t="s">
+      <c r="F278" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="F278" s="11">
+      <c r="G278" s="11">
         <v>2</v>
       </c>
-    </row>
-    <row r="279" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V278" s="1"/>
+      <c r="BN278" s="6"/>
+    </row>
+    <row r="279" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D279" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="E279" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="E279" s="11" t="s">
+      <c r="F279" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="F279" s="11">
+      <c r="G279" s="11">
         <v>1</v>
       </c>
-    </row>
-    <row r="282" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V279" s="1"/>
+      <c r="BN279" s="6"/>
+    </row>
+    <row r="282" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D282" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="283" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="283" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D283" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E283" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E283" s="11" t="s">
+      <c r="F283" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F283" s="11" t="s">
+      <c r="G283" s="11" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="284" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V283" s="1"/>
+      <c r="BN283" s="6"/>
+    </row>
+    <row r="284" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D284" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E284" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="E284" s="11" t="s">
+      <c r="F284" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="F284" s="11">
+      <c r="G284" s="11">
         <v>5</v>
       </c>
-    </row>
-    <row r="285" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V284" s="1"/>
+      <c r="BN284" s="6"/>
+    </row>
+    <row r="285" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D285" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="E285" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="E285" s="11" t="s">
+      <c r="F285" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="F285" s="11">
+      <c r="G285" s="11">
         <v>4</v>
       </c>
-    </row>
-    <row r="286" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V285" s="1"/>
+      <c r="BN285" s="6"/>
+    </row>
+    <row r="286" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D286" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="E286" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E286" s="11" t="s">
+      <c r="F286" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="F286" s="11">
+      <c r="G286" s="11">
         <v>3</v>
       </c>
-    </row>
-    <row r="287" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V286" s="1"/>
+      <c r="BN286" s="6"/>
+    </row>
+    <row r="287" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D287" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="E287" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E287" s="11" t="s">
+      <c r="F287" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="F287" s="11">
+      <c r="G287" s="11">
         <v>2</v>
       </c>
-    </row>
-    <row r="288" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V287" s="1"/>
+      <c r="BN287" s="6"/>
+    </row>
+    <row r="288" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D288" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E288" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="E288" s="11" t="s">
+      <c r="F288" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="F288" s="11">
+      <c r="G288" s="11">
         <v>1</v>
       </c>
-    </row>
-    <row r="291" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V288" s="1"/>
+      <c r="BN288" s="6"/>
+    </row>
+    <row r="291" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D291" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="292" spans="4:6" x14ac:dyDescent="0.25">
+    <row r="292" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D292" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="E292" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E292" s="11" t="s">
+      <c r="F292" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F292" s="11" t="s">
+      <c r="G292" s="11" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="293" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V292" s="1"/>
+      <c r="BN292" s="6"/>
+    </row>
+    <row r="293" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D293" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="E293" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="E293" s="11" t="s">
+      <c r="F293" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="F293" s="11">
+      <c r="G293" s="11">
         <v>5</v>
       </c>
-    </row>
-    <row r="294" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V293" s="1"/>
+      <c r="BN293" s="6"/>
+    </row>
+    <row r="294" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D294" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E294" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E294" s="11" t="s">
+      <c r="F294" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="F294" s="11">
+      <c r="G294" s="11">
         <v>4</v>
       </c>
-    </row>
-    <row r="295" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V294" s="1"/>
+      <c r="BN294" s="6"/>
+    </row>
+    <row r="295" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D295" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="E295" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E295" s="11" t="s">
+      <c r="F295" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F295" s="11">
+      <c r="G295" s="11">
         <v>3</v>
       </c>
-    </row>
-    <row r="296" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V295" s="1"/>
+      <c r="BN295" s="6"/>
+    </row>
+    <row r="296" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D296" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="E296" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="E296" s="11" t="s">
+      <c r="F296" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="F296" s="11">
+      <c r="G296" s="11">
         <v>2</v>
       </c>
-    </row>
-    <row r="297" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="V296" s="1"/>
+      <c r="BN296" s="6"/>
+    </row>
+    <row r="297" spans="4:66" x14ac:dyDescent="0.25">
       <c r="D297" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="E297" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="E297" s="11" t="s">
+      <c r="F297" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="F297" s="11">
+      <c r="G297" s="11">
         <v>1</v>
       </c>
+      <c r="V297" s="1"/>
+      <c r="BN297" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7804,6 +8091,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADQALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAxACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -7998,21 +8300,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADQALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAxACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAXABuACAAIAAgACAAUgBPAFcAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAIAAtACAAMQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAAsAFwAbgAgACAAQwBPAEwAVQBNAE4AKABUAGEAYgBsAGUASABlAGEAZABlAHIAQwBlAGwAbAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgAEEAcgByAGEAeQBEAGEAdABhACwAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsACAAWwBDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5AF0ALABcAG4AIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIABJAE4ARABFAFgAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAVQBOAEkAUQBVAEUAKABBAHIAcgBhAHkARABhAHQAYQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBPAFcAKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEMATwBMAFUATQBOACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQAsACAAMQAsACAAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsACAAXAAiAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AIAAgACAAIAApACwAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApACwAIAAwACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAWwBWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQBdACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBGAEYAYQBsAHMAZQApACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkAZgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkALAAgAFwAIgBcACIALAAgAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAEMAcgBpAHQAZQByAGkAYQAxACwAIABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACwAIABbAE0AdQBsAHQAaQBwAGwAaQBlAHIAXQAsACAAWwBDAHIAaQB0AGUAcgBpAGEAMgBdACwAWwBDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAXQAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABtAHUAbAB0AGkAcABsAGkAZQByACwAIABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsADEALABNAHUAbAB0AGkAcABsAGkAZQByACkALABcAG4AIAAgACAAIABxAHUAYQBuAHQAaQB0AHkALAAgAFEAdQBhAG4AdABpAHQAeQAqAE0AdQBsAHQAaQBwAGwAaQBlAHIALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADEAKQAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAyACwASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAHIAaQB0AGUAcgBpAGEAMgApACwAMQAsAC0ALQAoAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAyACkAKQAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABjAHIAaQB0AGUAcgBpAGEAMQAqAGMAcgBpAHQAZQByAGkAYQAyACoAcQB1AGEAbgB0AGkAdAB5ACkAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQAgAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAUwAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgACAAIAAgACAARQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAXABuACAAIAAgACAAIAAgACAAIABtACwATQBPAE4AVABIACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABkACwARABBAFkAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALAAgAC8AKgBoAGUAbABwAGUAcgA6ACAAZQBuAGQAIABkAGEAdABlACAAZgBvAHIAIABhACAAcgBlAHAAbwByAHQAaQBuAGcAIABwAGUAcgBpAG8AZAAgAHMAdABhAHIAdABpAG4AZwAgAGEAdAAgAGEAIABnAGkAdgBlAG4AIABkAGEAdABlACoALwBcAG4AIAAgACAAIAAgACAAIAAgAFAAZQByAGkAbwBkAEUAbgBkACwATABBAE0AQgBEAEEAKABzAHQALABFAEQAQQBUAEUAKABzAHQALAAxADIAKQAtADEAKQAsACAALwAqAG8AbgBsAHkAIABuAGUAZQBkACAAdABvACAAbABvAG8AawAgAGIAYQBjAGsAIAAzADYANQAgAGQAYQB5AHMAKABtAGEAeAAgAG8AdgBlAHIAbABhAHAAIAB3AGkAbgBkAG8AdwApACoALwBcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGEAIABlAG4AZABzACAAYgBlAGYAbwByAGUAIABTACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABuAGUAeAB0ACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjAFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAcAByAGUAdgBpAG8AdQBzACAAeQBlAGEAcgAqAC8AXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlAEUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbgAsAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AHIAcwAsAFMARQBRAFUARQBOAEMARQAoAG4ALAAxACwAZgBpAHIAcwB0AFkAZQBhAHIALAAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzACwARABBAFQARQAoAHkAcgBzACwAbQAsAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwAsAE0AQQBQACgAcwB0AGEAcgB0AHMALABQAGUAcgBpAG8AZABFAG4AZAApACwAXABuACAAIAAgACAAIAAgACAAIAB0AGEAZwAsAEkARgAoAHMAdABhAHIAdABzAD0AUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAIgAgACgAVABoAGkAcwAgAHIAZQBwAG8AcgB0AGkAbgBnACAAYwB5AGMAbABlACkAXAAiACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAHMAdABhAHIAdABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZQBuAGQAcwBUAGUAeAB0ACwAVABFAFgAVAAoAGUAbgBkAHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABuAD0AMAAsAFwAIgBcACIALABIAFMAVABBAEMASwAoAHMAdABhAHIAdABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAFwAIgAgAHQAbwAgAFwAIgAgAFwAdQAwADAAMgA2ACAAZQBuAGQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIAB0AGEAZwApACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAXABuAD0ATABBAE0AQgBEAEEAKABGAHUAbgBjAHQAaQBvAG4ALAAgAFQARQBYAFQAQgBFAEYATwBSAEUAKABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQAsACAAXAAiACgAXAAiACkAKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5ACwAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5ACwAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAPQBcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAgAD0AIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQA9AFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5AD0ASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAQQByAHIAYQB5AD0AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBMAG8AbwBrAHUAcAAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQALAAgAFwAbgAgACAAIAAgACAAIAAgACAAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABJAEYAKABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACAAKwAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABcAHUAMAAwADMAZQAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcAHUAMAAwADIANwBcACIAIABcAHUAMAAwADIANgAgAHMAaAAgAFwAdQAwADAAMgA2ACAAXAAiAFwAdQAwADAAMgA3ACEAXAAiACAAXAB1ADAAMAAyADYAIABhAGQAZAByAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAEQAaQBmAGYAZQByAGUAbgB0AFMAaABlAGUAdABcAG4APQBMAEEATQBCAEQAQQAoAFQAYQByAGcAZQB0AEMAZQBsAGwALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAcwBoACwAIABUAEUAWABUAEEARgBUAEUAUgAoAEMARQBMAEwAKABcACIAZgBpAGwAZQBuAGEAbQBlAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAIABcACIAXQBcACIAKQAsAFwAbgAgACAAIAAgAGEAZABkAHIALAAgAEMARQBMAEwAKABcACIAYQBkAGQAcgBlAHMAcwBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsAFwAbgAgACAAIAAgAFwAIgAjAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBVAE4ARAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAMAApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBJAE4AKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEEAWAAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABNAE0AUwAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFIAZQBzAHUAbAB0AHMASQB0AGUAbQBGAHIAbwBtAEUAcQB1AGEAdABpAG8AbgBUAGkAdABsAGUAQQBuAGQAUwBvAHUAcgBjAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGkAdABsAGUAQwBlAGwAbAAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAAsAFwAbgAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABMAEUARgBUACgAUwBvAHUAcgBjAGUAQwBlAGwAbAAsACAARgBJAE4ARAAoAFwAIgAsAFwAIgAsACAAUwBvAHUAcgBjAGUAQwBlAGwAbAApACAALQAxACkALAAgAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABcACIALAAgAFwAIgBcACIAKQAgAFwAdQAwADAAMgA2ACAAXAAiACAAXAAiACAAXAB1ADAAMAAyADYAIABUAGkAdABsAGUAQwBlAGwAbABcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -8023,6 +8310,25 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8041,25 +8347,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>

</xml_diff>